<commit_message>
Changed the CapEx source in the forecast sheet to take the adjusted capex from Statements
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8570968-7C2F-7742-AA71-196745752CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46326320-F300-6946-897C-CE5AA581779D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="3" activeTab="12" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -2287,9 +2287,6 @@
     <xf numFmtId="10" fontId="23" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="23" fillId="12" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2299,6 +2296,15 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2306,12 +2312,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -15388,12 +15388,12 @@
     <v>1</v>
     <v>Powered by Refinitiv</v>
     <v>317.39999999999998</v>
-    <v>199.26070000000001</v>
-    <v>1.1047</v>
-    <v>7.62</v>
-    <v>2.7046000000000001E-2</v>
-    <v>-0.3</v>
-    <v>-1.0369999999999999E-3</v>
+    <v>201.5</v>
+    <v>1.0868</v>
+    <v>14.25</v>
+    <v>4.8406999999999999E-2</v>
+    <v>-0.1893</v>
+    <v>-6.1339999999999995E-4</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15401,25 +15401,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>289.94</v>
+    <v>309.42</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46203.952167812502</v>
+    <v>46205.999965821095</v>
     <v>0</v>
-    <v>280.69499999999999</v>
-    <v>4249934489600</v>
+    <v>293.68</v>
+    <v>4532959916800</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>281.17</v>
-    <v>35.142899999999997</v>
-    <v>281.74</v>
-    <v>289.36</v>
-    <v>289.06</v>
+    <v>294.12</v>
+    <v>35.752499999999998</v>
+    <v>294.38</v>
+    <v>308.63</v>
+    <v>308.44069999999999</v>
     <v>14687360000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>65048942</v>
-    <v>63868052</v>
+    <v>75400626</v>
+    <v>64811799</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -15443,17 +15443,17 @@
     <v>Powered by Refinitiv</v>
     <v>46.87</v>
     <v>39.47</v>
-    <v>0.02</v>
-    <v>4.5750000000000001E-4</v>
+    <v>0.1</v>
+    <v>2.235E-3</v>
     <v>US</v>
-    <v>43.9</v>
+    <v>45.05</v>
     <v>Index</v>
     <v>3</v>
-    <v>43.67</v>
+    <v>44.53</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>43.78</v>
-    <v>43.72</v>
-    <v>43.74</v>
+    <v>45.03</v>
+    <v>44.75</v>
+    <v>44.85</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -15675,9 +15675,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq Last Sale</v>
+      <v>Source: Nasdaq</v>
       <v>GMT</v>
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>Delayed 15 minutes</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -16248,18 +16248,18 @@
   <sheetData>
     <row r="1" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="233" t="s">
+      <c r="B2" s="232" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="234"/>
-      <c r="E2" s="233" t="s">
+      <c r="C2" s="233"/>
+      <c r="E2" s="232" t="s">
         <v>286</v>
       </c>
-      <c r="F2" s="234"/>
-      <c r="H2" s="233" t="s">
+      <c r="F2" s="233"/>
+      <c r="H2" s="232" t="s">
         <v>327</v>
       </c>
-      <c r="I2" s="234"/>
+      <c r="I2" s="233"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="182" t="s">
@@ -16274,7 +16274,7 @@
       </c>
       <c r="F3" s="184">
         <f ca="1">Statement!AC143</f>
-        <v>4265166.4000000004</v>
+        <v>4549206.2</v>
       </c>
       <c r="H3" s="182" t="str">
         <f>'AVG target price'!B5</f>
@@ -16282,7 +16282,7 @@
       </c>
       <c r="I3" s="208">
         <f ca="1">'AVG target price'!C5</f>
-        <v>119.68851520308499</v>
+        <v>119.09057177167055</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16298,7 +16298,7 @@
       </c>
       <c r="F4" s="185">
         <f ca="1">Statement!AC144</f>
-        <v>4203282.4000000004</v>
+        <v>4487322.2</v>
       </c>
       <c r="H4" s="182" t="str">
         <f>'AVG target price'!B6</f>
@@ -16306,7 +16306,7 @@
       </c>
       <c r="I4" s="208">
         <f ca="1">'AVG target price'!C6</f>
-        <v>191.28349310124528</v>
+        <v>190.96664389474685</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16315,7 +16315,7 @@
       </c>
       <c r="C5" s="205" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
       <c r="E5" s="182" t="s">
         <v>242</v>
@@ -16339,14 +16339,14 @@
       </c>
       <c r="C6" s="205" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>289.06</v>
+        <v>308.44069999999999</v>
       </c>
       <c r="E6" s="182" t="s">
         <v>236</v>
       </c>
       <c r="F6" s="187">
         <f ca="1">Statement!AC140</f>
-        <v>34.989117291414757</v>
+        <v>37.319226118500609</v>
       </c>
       <c r="H6" s="182" t="str">
         <f>'AVG target price'!B8</f>
@@ -16354,7 +16354,7 @@
       </c>
       <c r="I6" s="208">
         <f ca="1">'AVG target price'!C8</f>
-        <v>122.21992262514725</v>
+        <v>122.01885943396663</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16363,14 +16363,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>7.62</v>
+        <v>14.25</v>
       </c>
       <c r="E7" s="183" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="188">
         <f ca="1">Statement!AC141</f>
-        <v>9.5100462960911933</v>
+        <v>10.143370156077635</v>
       </c>
       <c r="H7" s="181" t="str">
         <f>'AVG target price'!B9</f>
@@ -16378,7 +16378,7 @@
       </c>
       <c r="I7" s="209">
         <f ca="1">'AVG target price'!C9</f>
-        <v>142.9698408039568</v>
+        <v>142.69087684668344</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -16387,14 +16387,14 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-0.3</v>
+        <v>-0.1893</v>
       </c>
       <c r="E8" s="182" t="s">
         <v>264</v>
       </c>
       <c r="F8" s="189">
         <f ca="1">Statement!AC151</f>
-        <v>2.7126960392447993E-2</v>
+        <v>2.5433228328933518E-2</v>
       </c>
       <c r="H8" s="181" t="str">
         <f>'AVG target price'!B11</f>
@@ -16402,7 +16402,7 @@
       </c>
       <c r="I8" s="210">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.50591014375187726</v>
+        <v>-0.53766362036521587</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16411,14 +16411,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>2.7046000000000001E-2</v>
+        <v>4.8406999999999999E-2</v>
       </c>
       <c r="E9" s="182" t="s">
         <v>287</v>
       </c>
       <c r="F9" s="189">
         <f ca="1">Statement!AC152</f>
-        <v>2.8580315178324576E-2</v>
+        <v>2.6795839678579528E-2</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -16427,14 +16427,14 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-1.0369999999999999E-3</v>
+        <v>-6.1339999999999995E-4</v>
       </c>
       <c r="E10" s="182" t="s">
         <v>292</v>
       </c>
       <c r="F10" s="189">
         <f ca="1">Statement!AC154</f>
-        <v>1.8333634064077779E-2</v>
+        <v>1.7188932873607708E-2</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -16450,7 +16450,7 @@
       </c>
       <c r="F11" s="190">
         <f ca="1">Statement!AC153</f>
-        <v>3.5941387890517005E-3</v>
+        <v>3.3697307455529276E-3</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16459,7 +16459,7 @@
       </c>
       <c r="C12" s="206" cm="1">
         <f t="array" aca="1" ref="C12" ca="1">_FV(C3,"52 week low",TRUE)</f>
-        <v>199.26070000000001</v>
+        <v>201.5</v>
       </c>
       <c r="E12" s="182" t="s">
         <v>99</v>
@@ -16475,7 +16475,7 @@
       </c>
       <c r="C13" s="206" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.1047</v>
+        <v>1.0868</v>
       </c>
       <c r="E13" s="182" t="s">
         <v>101</v>
@@ -16491,7 +16491,7 @@
       </c>
       <c r="C14" s="207" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>63868052</v>
+        <v>64811799</v>
       </c>
       <c r="E14" s="183" t="s">
         <v>102</v>
@@ -16507,7 +16507,7 @@
       </c>
       <c r="F15" s="189">
         <f ca="1">Statement!AC166</f>
-        <v>1.4509164284891674E-2</v>
+        <v>1.3603252365214836E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16520,10 +16520,10 @@
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="235" t="s">
+      <c r="B17" s="234" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="235"/>
+      <c r="C17" s="234"/>
       <c r="E17" s="181" t="s">
         <v>295</v>
       </c>
@@ -16596,14 +16596,14 @@
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="235" t="s">
+      <c r="B25" s="234" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="235"/>
-      <c r="E25" s="233" t="s">
+      <c r="C25" s="234"/>
+      <c r="E25" s="232" t="s">
         <v>342</v>
       </c>
-      <c r="F25" s="234"/>
+      <c r="F25" s="233"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="181" t="s">
@@ -16617,7 +16617,7 @@
       </c>
       <c r="F26" s="216" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>43.74</v>
+        <v>44.85</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="F27" s="217">
         <f ca="1">F26/1000</f>
-        <v>4.3740000000000001E-2</v>
+        <v>4.4850000000000001E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -16652,15 +16652,15 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B33" s="232" t="s">
+      <c r="B33" s="235" t="s">
         <v>337</v>
       </c>
-      <c r="C33" s="232"/>
-      <c r="D33" s="232"/>
-      <c r="E33" s="232"/>
-      <c r="F33" s="232"/>
-      <c r="G33" s="232"/>
-      <c r="H33" s="232"/>
+      <c r="C33" s="235"/>
+      <c r="D33" s="235"/>
+      <c r="E33" s="235"/>
+      <c r="F33" s="235"/>
+      <c r="G33" s="235"/>
+      <c r="H33" s="235"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
@@ -16673,24 +16673,24 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="232"/>
-      <c r="C39" s="232"/>
-      <c r="D39" s="232"/>
-      <c r="E39" s="232"/>
-      <c r="F39" s="232"/>
-      <c r="G39" s="232"/>
-      <c r="H39" s="232"/>
+      <c r="B39" s="235"/>
+      <c r="C39" s="235"/>
+      <c r="D39" s="235"/>
+      <c r="E39" s="235"/>
+      <c r="F39" s="235"/>
+      <c r="G39" s="235"/>
+      <c r="H39" s="235"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B42" s="232" t="s">
+      <c r="B42" s="235" t="s">
         <v>340</v>
       </c>
-      <c r="C42" s="232"/>
-      <c r="D42" s="232"/>
-      <c r="E42" s="232"/>
-      <c r="F42" s="232"/>
-      <c r="G42" s="232"/>
-      <c r="H42" s="232"/>
+      <c r="C42" s="235"/>
+      <c r="D42" s="235"/>
+      <c r="E42" s="235"/>
+      <c r="F42" s="235"/>
+      <c r="G42" s="235"/>
+      <c r="H42" s="235"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="41" t="s">
@@ -16705,24 +16705,24 @@
       </c>
     </row>
     <row r="49" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="232"/>
-      <c r="C49" s="232"/>
-      <c r="D49" s="232"/>
-      <c r="E49" s="232"/>
-      <c r="F49" s="232"/>
-      <c r="G49" s="232"/>
-      <c r="H49" s="232"/>
+      <c r="B49" s="235"/>
+      <c r="C49" s="235"/>
+      <c r="D49" s="235"/>
+      <c r="E49" s="235"/>
+      <c r="F49" s="235"/>
+      <c r="G49" s="235"/>
+      <c r="H49" s="235"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="232" t="s">
+      <c r="B52" s="235" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="232"/>
-      <c r="D52" s="232"/>
-      <c r="E52" s="232"/>
-      <c r="F52" s="232"/>
-      <c r="G52" s="232"/>
-      <c r="H52" s="232"/>
+      <c r="C52" s="235"/>
+      <c r="D52" s="235"/>
+      <c r="E52" s="235"/>
+      <c r="F52" s="235"/>
+      <c r="G52" s="235"/>
+      <c r="H52" s="235"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" s="41" t="s">
@@ -16737,28 +16737,28 @@
       </c>
     </row>
     <row r="59" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="232"/>
-      <c r="C59" s="232"/>
-      <c r="D59" s="232"/>
-      <c r="E59" s="232"/>
-      <c r="F59" s="232"/>
-      <c r="G59" s="232"/>
-      <c r="H59" s="232"/>
+      <c r="B59" s="235"/>
+      <c r="C59" s="235"/>
+      <c r="D59" s="235"/>
+      <c r="E59" s="235"/>
+      <c r="F59" s="235"/>
+      <c r="G59" s="235"/>
+      <c r="H59" s="235"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B52:H52"/>
+    <mergeCell ref="B59:H59"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B39:H39"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B49:H49"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="E25:F25"/>
-    <mergeCell ref="B52:H52"/>
-    <mergeCell ref="B59:H59"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B49:H49"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C10">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
@@ -16828,36 +16828,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="232" t="s">
+      <c r="C2" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
+      <c r="I2" s="235"/>
+      <c r="J2" s="235"/>
+      <c r="K2" s="235"/>
+      <c r="L2" s="235"/>
       <c r="O2" s="5"/>
-      <c r="S2" s="232" t="s">
+      <c r="S2" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="232"/>
-      <c r="U2" s="232"/>
-      <c r="V2" s="232"/>
-      <c r="W2" s="232"/>
-      <c r="X2" s="232"/>
-      <c r="Y2" s="232"/>
-      <c r="Z2" s="232"/>
-      <c r="AA2" s="232" t="s">
+      <c r="T2" s="235"/>
+      <c r="U2" s="235"/>
+      <c r="V2" s="235"/>
+      <c r="W2" s="235"/>
+      <c r="X2" s="235"/>
+      <c r="Y2" s="235"/>
+      <c r="Z2" s="235"/>
+      <c r="AA2" s="235" t="s">
         <v>111</v>
       </c>
-      <c r="AB2" s="232"/>
-      <c r="AC2" s="232"/>
+      <c r="AB2" s="235"/>
+      <c r="AC2" s="235"/>
       <c r="AE2" s="85" t="s">
         <v>112</v>
       </c>
@@ -18228,35 +18228,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="232" t="s">
+      <c r="C2" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
-      <c r="P2" s="232" t="s">
+      <c r="I2" s="235"/>
+      <c r="J2" s="235"/>
+      <c r="K2" s="235"/>
+      <c r="L2" s="235"/>
+      <c r="P2" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="Q2" s="232"/>
-      <c r="R2" s="232"/>
-      <c r="S2" s="232"/>
-      <c r="T2" s="232"/>
-      <c r="U2" s="232"/>
-      <c r="V2" s="232"/>
-      <c r="W2" s="232"/>
-      <c r="X2" s="232" t="s">
+      <c r="Q2" s="235"/>
+      <c r="R2" s="235"/>
+      <c r="S2" s="235"/>
+      <c r="T2" s="235"/>
+      <c r="U2" s="235"/>
+      <c r="V2" s="235"/>
+      <c r="W2" s="235"/>
+      <c r="X2" s="235" t="s">
         <v>111</v>
       </c>
-      <c r="Y2" s="232"/>
-      <c r="Z2" s="232"/>
+      <c r="Y2" s="235"/>
+      <c r="Z2" s="235"/>
       <c r="AB2" s="85" t="s">
         <v>112</v>
       </c>
@@ -19487,20 +19487,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="232" t="s">
+      <c r="C3" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="232"/>
-      <c r="E3" s="232"/>
-      <c r="F3" s="232"/>
+      <c r="D3" s="235"/>
+      <c r="E3" s="235"/>
+      <c r="F3" s="235"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="232"/>
-      <c r="J3" s="232"/>
-      <c r="K3" s="232"/>
-      <c r="L3" s="232"/>
+      <c r="I3" s="235"/>
+      <c r="J3" s="235"/>
+      <c r="K3" s="235"/>
+      <c r="L3" s="235"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -20811,23 +20811,23 @@
         <v>58</v>
       </c>
       <c r="C45" s="114">
-        <f>-Statement!M59</f>
+        <f>-Statement!M108</f>
         <v>11085</v>
       </c>
       <c r="D45" s="114">
-        <f>-Statement!N59</f>
+        <f>-Statement!N108</f>
         <v>10708</v>
       </c>
       <c r="E45" s="114">
-        <f>-Statement!O59</f>
+        <f>-Statement!O108</f>
         <v>10959</v>
       </c>
       <c r="F45" s="114">
-        <f>-Statement!P59</f>
+        <f>-Statement!P108</f>
         <v>9447</v>
       </c>
       <c r="G45" s="115">
-        <f>-Statement!Q59</f>
+        <f>-Statement!Q108</f>
         <v>12715</v>
       </c>
       <c r="H45" s="25">
@@ -20893,6 +20893,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -20900,12 +20906,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -20943,20 +20943,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="232" t="s">
+      <c r="C2" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
+      <c r="I2" s="235"/>
+      <c r="J2" s="235"/>
+      <c r="K2" s="235"/>
+      <c r="L2" s="235"/>
       <c r="S2" s="246"/>
       <c r="T2" s="246"/>
       <c r="U2" s="246"/>
@@ -21965,16 +21965,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AA2:AC2"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="S4:AC4"/>
+    <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C18:L18"/>
     <mergeCell ref="C31:L31"/>
     <mergeCell ref="C25:L25"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="AA2:AC2"/>
-    <mergeCell ref="C4:L4"/>
-    <mergeCell ref="S4:AC4"/>
-    <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C18:L18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22037,10 +22037,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="232" t="s">
+      <c r="B4" s="235" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="232"/>
+      <c r="C4" s="235"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -22057,7 +22057,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22066,7 +22066,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4265166.4000000004</v>
+        <v>4549206.2</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22084,7 +22084,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>4.3740000000000001E-2</v>
+        <v>4.4850000000000001E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22093,7 +22093,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.1047</v>
+        <v>1.0868</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22125,10 +22125,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="232" t="s">
+      <c r="B15" s="235" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="232"/>
+      <c r="C15" s="235"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -22136,7 +22136,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.9474341966511516E-2</v>
+        <v>1.8280646015858892E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22145,7 +22145,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98052565803348846</v>
+        <v>0.98171935398414112</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22163,7 +22163,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>9.3451499999999993E-2</v>
+        <v>9.3756000000000006E-2</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22172,7 +22172,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.2346983483856337E-2</v>
+        <v>9.2713619283529725E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22217,20 +22217,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="232" t="s">
+      <c r="C3" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="232"/>
-      <c r="E3" s="232"/>
-      <c r="F3" s="232"/>
+      <c r="D3" s="235"/>
+      <c r="E3" s="235"/>
+      <c r="F3" s="235"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="232"/>
-      <c r="J3" s="232"/>
-      <c r="K3" s="232"/>
-      <c r="L3" s="232"/>
+      <c r="I3" s="235"/>
+      <c r="J3" s="235"/>
+      <c r="K3" s="235"/>
+      <c r="L3" s="235"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -22423,7 +22423,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1938098.253247638</v>
+        <v>1928325.9958641303</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22477,23 +22477,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>96445.519730698827</v>
+        <v>96413.15957738203</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>93256.520813370589</v>
+        <v>93193.951001053298</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>90487.615543884356</v>
+        <v>90396.562769008087</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>87590.239245136399</v>
+        <v>87472.742554731027</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88387.932974733514</v>
+        <v>88239.749402833404</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22512,14 +22512,14 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1246156.8857856491</v>
+        <v>1237794.8626094162</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="232" t="s">
+      <c r="B13" s="235" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="232"/>
+      <c r="C13" s="235"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -22535,14 +22535,14 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2346983483856337E-2</v>
+        <v>9.2713619283529725E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="232" t="s">
+      <c r="B18" s="235" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="232"/>
+      <c r="C18" s="235"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -22550,7 +22550,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>456167.82830782369</v>
+        <v>455716.16530500783</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22559,7 +22559,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1246156.8857856491</v>
+        <v>1237794.8626094162</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22568,7 +22568,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1702324.7140934728</v>
+        <v>1693511.027914424</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22595,7 +22595,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1764208.7140934728</v>
+        <v>1755395.027914424</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22613,7 +22613,7 @@
       </c>
       <c r="C26" s="142">
         <f ca="1">C24/C25</f>
-        <v>119.68851520308499</v>
+        <v>119.09057177167055</v>
       </c>
     </row>
   </sheetData>
@@ -22656,20 +22656,20 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="232" t="s">
+      <c r="C2" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
+      <c r="I2" s="235"/>
+      <c r="J2" s="235"/>
+      <c r="K2" s="235"/>
+      <c r="L2" s="235"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -23601,10 +23601,10 @@
       <c r="N36" s="91"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B37" s="232" t="s">
+      <c r="B37" s="235" t="s">
         <v>202</v>
       </c>
-      <c r="C37" s="232"/>
+      <c r="C37" s="235"/>
       <c r="N37" s="91"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
@@ -23622,7 +23622,7 @@
       </c>
       <c r="C39" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2346983483856337E-2</v>
+        <v>9.2713619283529725E-2</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -23657,7 +23657,7 @@
       </c>
       <c r="C43" s="24">
         <f ca="1">C42/(1+C39)^5-G30+G31</f>
-        <v>2819518.6883123554</v>
+        <v>2814848.3310085684</v>
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.2">
@@ -23675,14 +23675,14 @@
       </c>
       <c r="C45" s="142">
         <f ca="1">C43/C44</f>
-        <v>191.28349310124528</v>
+        <v>190.96664389474685</v>
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B47" s="232" t="s">
+      <c r="B47" s="235" t="s">
         <v>207</v>
       </c>
-      <c r="C47" s="232"/>
+      <c r="C47" s="235"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B48" s="1" t="s">
@@ -23738,10 +23738,10 @@
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B55" s="232" t="s">
+      <c r="B55" s="235" t="s">
         <v>321</v>
       </c>
-      <c r="C55" s="232"/>
+      <c r="C55" s="235"/>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B56" s="1" t="s">
@@ -23758,7 +23758,7 @@
       </c>
       <c r="C57" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2346983483856337E-2</v>
+        <v>9.2713619283529725E-2</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.2">
@@ -23784,7 +23784,7 @@
       </c>
       <c r="C60" s="24">
         <f ca="1">C59/(1+C57)^5-G30+G31</f>
-        <v>1801521.6594946703</v>
+        <v>1798557.9880566681</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.2">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="C62" s="142">
         <f ca="1">C60/C61</f>
-        <v>122.21992262514725</v>
+        <v>122.01885943396663</v>
       </c>
     </row>
   </sheetData>
@@ -23854,10 +23854,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="232" t="s">
+      <c r="B4" s="235" t="s">
         <v>212</v>
       </c>
-      <c r="C4" s="232"/>
+      <c r="C4" s="235"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -23866,7 +23866,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>119.68851520308499</v>
+        <v>119.09057177167055</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -23875,7 +23875,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C45</f>
-        <v>191.28349310124528</v>
+        <v>190.96664389474685</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -23893,7 +23893,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C62</f>
-        <v>122.21992262514725</v>
+        <v>122.01885943396663</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="C9" s="142">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>142.9698408039568</v>
+        <v>142.69087684668344</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -23911,7 +23911,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C5</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -23920,7 +23920,7 @@
       </c>
       <c r="C11" s="151">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.50591014375187726</v>
+        <v>-0.53766362036521587</v>
       </c>
     </row>
   </sheetData>
@@ -23985,20 +23985,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="232" t="s">
+      <c r="C3" s="235" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="232"/>
-      <c r="E3" s="232"/>
-      <c r="F3" s="232"/>
+      <c r="D3" s="235"/>
+      <c r="E3" s="235"/>
+      <c r="F3" s="235"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="232"/>
-      <c r="J3" s="232"/>
-      <c r="K3" s="232"/>
-      <c r="L3" s="232"/>
+      <c r="I3" s="235"/>
+      <c r="J3" s="235"/>
+      <c r="K3" s="235"/>
+      <c r="L3" s="235"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -24173,7 +24173,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>5282338.0052034836</v>
+        <v>5255703.4594641058</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -24227,23 +24227,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>145077.1746060657</v>
+        <v>145028.49718044625</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>164687.31935137906</v>
+        <v>164576.82354290391</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>186948.17588492756</v>
+        <v>186760.06008510161</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>212218.04207118601</v>
+        <v>211933.36517336537</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>240903.64705269467</v>
+        <v>240499.76881159769</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -24262,7 +24262,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3396433.5230172998</v>
+        <v>3373642.6078765481</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -24278,7 +24278,7 @@
       </c>
       <c r="C15" s="153">
         <f ca="1">Overview!C5</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -24287,7 +24287,7 @@
       </c>
       <c r="C16" s="153">
         <f ca="1">C36</f>
-        <v>300.13970735913074</v>
+        <v>298.51740468917842</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -24326,7 +24326,7 @@
       </c>
       <c r="C21" s="219">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2346983483856337E-2</v>
+        <v>9.2713619283529725E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -24344,7 +24344,7 @@
       </c>
       <c r="C23" s="158">
         <f ca="1">C15*C22</f>
-        <v>4249830.32</v>
+        <v>4532848.8099999996</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="C26" s="159">
         <f ca="1">C23+C25-C24</f>
-        <v>4187946.3200000003</v>
+        <v>4470964.8099999996</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -24387,7 +24387,7 @@
       </c>
       <c r="C29" s="158">
         <f ca="1">SUM(H10:L10)</f>
-        <v>949834.35896625312</v>
+        <v>948798.51479341486</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -24396,7 +24396,7 @@
       </c>
       <c r="C30" s="158">
         <f ca="1">L11</f>
-        <v>3396433.5230172998</v>
+        <v>3373642.6078765481</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="C31" s="161">
         <f ca="1">C29+C30</f>
-        <v>4346267.8819835531</v>
+        <v>4322441.1226699632</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -24432,7 +24432,7 @@
       </c>
       <c r="C34" s="161">
         <f ca="1">C31+C32-C33</f>
-        <v>4408151.8819835531</v>
+        <v>4384325.1226699632</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -24450,7 +24450,7 @@
       </c>
       <c r="C36" s="164">
         <f ca="1">C34/C35</f>
-        <v>300.13970735913074</v>
+        <v>298.51740468917842</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -24897,17 +24897,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C39:L39"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C39:L39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -31305,7 +31305,7 @@
       <c r="AA114" s="68"/>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31352,7 +31352,7 @@
       <c r="AA115" s="68"/>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32266,7 +32266,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>34.989117291414757</v>
+        <v>37.319226118500609</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32303,7 +32303,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>9.5100462960911933</v>
+        <v>10.143370156077635</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32340,7 +32340,7 @@
       <c r="AA142" s="49"/>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>39.907882544064755</v>
+        <v>42.565557746664034</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32377,7 +32377,7 @@
       <c r="AA143" s="49"/>
       <c r="AC143" s="143">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4265166.4000000004</v>
+        <v>4549206.2</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -32414,7 +32414,7 @@
       <c r="AA144" s="49"/>
       <c r="AC144" s="143">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4203282.4000000004</v>
+        <v>4487322.2</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -32451,7 +32451,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="180">
         <f ca="1">AC144/AC5</f>
-        <v>9.3107916410081479</v>
+        <v>9.9399750134015008</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -32488,7 +32488,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="180">
         <f ca="1">AC144/AC11</f>
-        <v>28.522742016475988</v>
+        <v>30.450186610208597</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -32623,7 +32623,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="89">AC143/AC147</f>
-        <v>36.863695214388812</v>
+        <v>39.318642016922929</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -32660,7 +32660,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="89"/>
-        <v>36.366972692027488</v>
+        <v>38.824496757041281</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -32697,7 +32697,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="92">AC147/AC143</f>
-        <v>2.7126960392447993E-2</v>
+        <v>2.5433228328933518E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -32734,7 +32734,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.8580315178324576E-2</v>
+        <v>2.6795839678579528E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -32771,7 +32771,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="151">
         <f ca="1">AC81/AC115</f>
-        <v>3.5941387890517005E-3</v>
+        <v>3.3697307455529276E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -32808,7 +32808,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="151">
         <f ca="1">-AC62/AC143</f>
-        <v>1.8333634064077779E-2</v>
+        <v>1.7188932873607708E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -32845,7 +32845,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="151">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>2.1979447273147417E-2</v>
+        <v>2.0607111631915035E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33348,7 +33348,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="151">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.4509164284891674E-2</v>
+        <v>1.3603252365214836E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35345,15 +35345,15 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="232" t="s">
+      <c r="B4" s="235" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="232"/>
-      <c r="E4" s="232" t="s">
+      <c r="C4" s="235"/>
+      <c r="E4" s="235" t="s">
         <v>239</v>
       </c>
-      <c r="F4" s="232"/>
-      <c r="G4" s="232"/>
+      <c r="F4" s="235"/>
+      <c r="G4" s="235"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
@@ -35361,7 +35361,7 @@
       </c>
       <c r="C5" s="169">
         <f ca="1">Overview!C5</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -35377,7 +35377,7 @@
       </c>
       <c r="C6" s="170">
         <f ca="1">Statement!AC143</f>
-        <v>4265166.4000000004</v>
+        <v>4549206.2</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -35397,7 +35397,7 @@
       </c>
       <c r="C7" s="170">
         <f ca="1">Statement!AC144</f>
-        <v>4203282.4000000004</v>
+        <v>4487322.2</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -35417,7 +35417,7 @@
       </c>
       <c r="C8" s="171">
         <f ca="1">Statement!AC140</f>
-        <v>34.989117291414757</v>
+        <v>37.319226118500609</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>242</v>
@@ -35437,7 +35437,7 @@
       </c>
       <c r="C9" s="171">
         <f ca="1">Statement!AC141</f>
-        <v>9.5100462960911933</v>
+        <v>10.143370156077635</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>243</v>
@@ -35457,7 +35457,7 @@
       </c>
       <c r="C10" s="171">
         <f ca="1">Statement!AC142</f>
-        <v>39.907882544064755</v>
+        <v>42.565557746664034</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -35477,7 +35477,7 @@
       </c>
       <c r="C11" s="171">
         <f ca="1">Statement!AC145</f>
-        <v>9.3107916410081479</v>
+        <v>9.9399750134015008</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -35486,18 +35486,18 @@
       </c>
       <c r="C12" s="171">
         <f ca="1">Statement!AC146</f>
-        <v>28.522742016475988</v>
+        <v>30.450186610208597</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="232" t="s">
+      <c r="B15" s="235" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="232"/>
-      <c r="E15" s="232" t="s">
+      <c r="C15" s="235"/>
+      <c r="E15" s="235" t="s">
         <v>245</v>
       </c>
-      <c r="F15" s="232"/>
+      <c r="F15" s="235"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
@@ -35548,14 +35548,14 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="232" t="s">
+      <c r="B21" s="235" t="s">
         <v>244</v>
       </c>
-      <c r="C21" s="232"/>
-      <c r="E21" s="232" t="s">
+      <c r="C21" s="235"/>
+      <c r="E21" s="235" t="s">
         <v>248</v>
       </c>
-      <c r="F21" s="232"/>
+      <c r="F21" s="235"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
@@ -35624,14 +35624,14 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B29" s="232" t="s">
+      <c r="B29" s="235" t="s">
         <v>249</v>
       </c>
-      <c r="C29" s="232"/>
-      <c r="E29" s="232" t="s">
+      <c r="C29" s="235"/>
+      <c r="E29" s="235" t="s">
         <v>255</v>
       </c>
-      <c r="F29" s="232"/>
+      <c r="F29" s="235"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -35707,14 +35707,14 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B37" s="232" t="s">
+      <c r="B37" s="235" t="s">
         <v>267</v>
       </c>
-      <c r="C37" s="232"/>
-      <c r="E37" s="232" t="s">
+      <c r="C37" s="235"/>
+      <c r="E37" s="235" t="s">
         <v>270</v>
       </c>
-      <c r="F37" s="232"/>
+      <c r="F37" s="235"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
@@ -35722,7 +35722,7 @@
       </c>
       <c r="C38" s="172">
         <f ca="1">Statement!AC152</f>
-        <v>2.8580315178324576E-2</v>
+        <v>2.6795839678579528E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>269</v>
@@ -35738,7 +35738,7 @@
       </c>
       <c r="C39" s="212">
         <f ca="1">Statement!AC151</f>
-        <v>2.7126960392447993E-2</v>
+        <v>2.5433228328933518E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>271</v>
@@ -35754,7 +35754,7 @@
       </c>
       <c r="C40" s="172">
         <f ca="1">Statement!AC153</f>
-        <v>3.5941387890517005E-3</v>
+        <v>3.3697307455529276E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>272</v>
@@ -35770,7 +35770,7 @@
       </c>
       <c r="C41" s="172">
         <f ca="1">Statement!AC154</f>
-        <v>1.8333634064077779E-2</v>
+        <v>1.7188932873607708E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -35779,18 +35779,18 @@
       </c>
       <c r="C42" s="172">
         <f ca="1">Statement!AC155</f>
-        <v>2.1979447273147417E-2</v>
+        <v>2.0607111631915035E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B45" s="232" t="s">
+      <c r="B45" s="235" t="s">
         <v>278</v>
       </c>
-      <c r="C45" s="232"/>
-      <c r="E45" s="232" t="s">
+      <c r="C45" s="235"/>
+      <c r="E45" s="235" t="s">
         <v>284</v>
       </c>
-      <c r="F45" s="232"/>
+      <c r="F45" s="235"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
@@ -35823,18 +35823,18 @@
       </c>
       <c r="F48" s="172">
         <f ca="1">Statement!AC166</f>
-        <v>1.4509164284891674E-2</v>
+        <v>1.3603252365214836E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B51" s="232" t="s">
+      <c r="B51" s="235" t="s">
         <v>281</v>
       </c>
-      <c r="C51" s="232"/>
-      <c r="E51" s="232" t="s">
+      <c r="C51" s="235"/>
+      <c r="E51" s="235" t="s">
         <v>302</v>
       </c>
-      <c r="F51" s="232"/>
+      <c r="F51" s="235"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
@@ -36002,7 +36002,7 @@
       </c>
       <c r="I6" s="169">
         <f ca="1">Statement!AC114</f>
-        <v>289.36</v>
+        <v>308.63</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36031,7 +36031,7 @@
       </c>
       <c r="I7" s="170">
         <f ca="1">Statement!AC143</f>
-        <v>4265166.4000000004</v>
+        <v>4549206.2</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36060,7 +36060,7 @@
       </c>
       <c r="I8" s="170">
         <f ca="1">Statement!AC144</f>
-        <v>4203282.4000000004</v>
+        <v>4487322.2</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36089,7 +36089,7 @@
       </c>
       <c r="I9" s="171">
         <f ca="1">Statement!AC140</f>
-        <v>34.989117291414757</v>
+        <v>37.319226118500609</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36118,7 +36118,7 @@
       </c>
       <c r="I10" s="171">
         <f ca="1">Statement!AC141</f>
-        <v>9.5100462960911933</v>
+        <v>10.143370156077635</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="I11" s="171">
         <f ca="1">Statement!AC142</f>
-        <v>39.907882544064755</v>
+        <v>42.565557746664034</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36176,7 +36176,7 @@
       </c>
       <c r="I12" s="171">
         <f ca="1">Statement!AC145</f>
-        <v>9.3107916410081479</v>
+        <v>9.9399750134015008</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36205,7 +36205,7 @@
       </c>
       <c r="I13" s="171">
         <f ca="1">Statement!AC146</f>
-        <v>28.522742016475988</v>
+        <v>30.450186610208597</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -36978,7 +36978,7 @@
       </c>
       <c r="I51" s="172">
         <f ca="1">Statement!AC152</f>
-        <v>2.8580315178324576E-2</v>
+        <v>2.6795839678579528E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37007,7 +37007,7 @@
       </c>
       <c r="I52" s="172">
         <f ca="1">Statement!AC151</f>
-        <v>2.7126960392447993E-2</v>
+        <v>2.5433228328933518E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37036,7 +37036,7 @@
       </c>
       <c r="I53" s="172">
         <f ca="1">Statement!AC153</f>
-        <v>3.5941387890517005E-3</v>
+        <v>3.3697307455529276E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37065,7 +37065,7 @@
       </c>
       <c r="I54" s="172">
         <f ca="1">Statement!AC154</f>
-        <v>1.8333634064077779E-2</v>
+        <v>1.7188932873607708E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37094,7 +37094,7 @@
       </c>
       <c r="I55" s="172">
         <f ca="1">Statement!AC155</f>
-        <v>2.1979447273147417E-2</v>
+        <v>2.0607111631915035E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37330,7 +37330,7 @@
       </c>
       <c r="I68" s="193">
         <f ca="1">Statement!AC166</f>
-        <v>1.4509164284891674E-2</v>
+        <v>1.3603252365214836E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38022,14 +38022,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="236" t="s">
+      <c r="C3" s="238" t="s">
         <v>312</v>
       </c>
-      <c r="D3" s="237"/>
-      <c r="F3" s="238" t="s">
+      <c r="D3" s="239"/>
+      <c r="F3" s="240" t="s">
         <v>313</v>
       </c>
-      <c r="G3" s="237"/>
+      <c r="G3" s="239"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38096,19 +38096,19 @@
       <c r="B7" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C7" s="239">
+      <c r="C7" s="236">
         <f>Statement!AA88</f>
         <v>-0.22657836890286318</v>
       </c>
-      <c r="D7" s="240"/>
-      <c r="F7" s="239">
+      <c r="D7" s="237"/>
+      <c r="F7" s="236">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16595182415922985</v>
       </c>
-      <c r="G7" s="240"/>
+      <c r="G7" s="237"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="204" t="s">
@@ -38135,19 +38135,19 @@
       <c r="B9" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C9" s="239">
+      <c r="C9" s="236">
         <f>Statement!AA89</f>
         <v>-0.24316672257631666</v>
       </c>
-      <c r="D9" s="240"/>
-      <c r="F9" s="239">
+      <c r="D9" s="237"/>
+      <c r="F9" s="236">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>0.11706805038421929</v>
       </c>
-      <c r="G9" s="240"/>
+      <c r="G9" s="237"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="204" t="s">
@@ -38174,19 +38174,19 @@
       <c r="B11" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C11" s="239">
+      <c r="C11" s="236">
         <f>Statement!AA90</f>
         <v>-0.2087215264838006</v>
       </c>
-      <c r="D11" s="240"/>
-      <c r="F11" s="239">
+      <c r="D11" s="237"/>
+      <c r="F11" s="236">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.22096418302984375</v>
       </c>
-      <c r="G11" s="240"/>
+      <c r="G11" s="237"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="204" t="s">
@@ -38213,19 +38213,19 @@
       <c r="B13" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C13" s="239">
+      <c r="C13" s="236">
         <f>Statement!AA93</f>
         <v>2.8129930899396048E-2</v>
       </c>
-      <c r="D13" s="240"/>
-      <c r="F13" s="239">
+      <c r="D13" s="237"/>
+      <c r="F13" s="236">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.23681110092944102</v>
       </c>
-      <c r="G13" s="240"/>
+      <c r="G13" s="237"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="204" t="s">
@@ -38252,19 +38252,19 @@
       <c r="B15" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C15" s="239">
+      <c r="C15" s="236">
         <f>Statement!AA94</f>
         <v>-0.29432470699284197</v>
       </c>
-      <c r="D15" s="240"/>
-      <c r="F15" s="239">
+      <c r="D15" s="237"/>
+      <c r="F15" s="236">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.21278177701172732</v>
       </c>
-      <c r="G15" s="240"/>
+      <c r="G15" s="237"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="204" t="s">
@@ -38291,19 +38291,19 @@
       <c r="B17" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C17" s="239">
+      <c r="C17" s="236">
         <f>Statement!AA96</f>
         <v>-0.29738461173005204</v>
       </c>
-      <c r="D17" s="240"/>
-      <c r="F17" s="239">
+      <c r="D17" s="237"/>
+      <c r="F17" s="236">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.19362389023405974</v>
       </c>
-      <c r="G17" s="240"/>
+      <c r="G17" s="237"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="204" t="s">
@@ -38330,22 +38330,22 @@
       <c r="B19" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C19" s="239">
+      <c r="C19" s="236">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-5.6718433490884537E-3</v>
       </c>
-      <c r="D19" s="240"/>
-      <c r="F19" s="239">
+      <c r="D19" s="237"/>
+      <c r="F19" s="236">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-2.1918172157279491E-2</v>
       </c>
-      <c r="G19" s="240"/>
+      <c r="G19" s="237"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="204" t="s">
@@ -38372,22 +38372,22 @@
       <c r="B21" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C21" s="239">
+      <c r="C21" s="236">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>-0.29225352112676062</v>
       </c>
-      <c r="D21" s="240"/>
-      <c r="F21" s="239">
+      <c r="D21" s="237"/>
+      <c r="F21" s="236">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.21818181818181812</v>
       </c>
-      <c r="G21" s="240"/>
+      <c r="G21" s="237"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -38435,22 +38435,22 @@
       <c r="B25" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C25" s="239">
+      <c r="C25" s="236">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>-0.22956141399989749</v>
       </c>
-      <c r="D25" s="240"/>
-      <c r="F25" s="239">
+      <c r="D25" s="237"/>
+      <c r="F25" s="236">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11851668113605358</v>
       </c>
-      <c r="G25" s="240"/>
+      <c r="G25" s="237"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -38477,22 +38477,22 @@
       <c r="B27" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C27" s="239">
+      <c r="C27" s="236">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>-0.26453625543962672</v>
       </c>
-      <c r="D27" s="240"/>
-      <c r="F27" s="239">
+      <c r="D27" s="237"/>
+      <c r="F27" s="236">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.14725607262615523</v>
       </c>
-      <c r="G27" s="240"/>
+      <c r="G27" s="237"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -38519,22 +38519,22 @@
       <c r="B29" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C29" s="239">
+      <c r="C29" s="236">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-0.19701480843061975</v>
       </c>
-      <c r="D29" s="240"/>
-      <c r="F29" s="239">
+      <c r="D29" s="237"/>
+      <c r="F29" s="236">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.28090238720159982</v>
       </c>
-      <c r="G29" s="240"/>
+      <c r="G29" s="237"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -38561,22 +38561,22 @@
       <c r="B31" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C31" s="239">
+      <c r="C31" s="236">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.10751088919579305</v>
       </c>
-      <c r="D31" s="240"/>
-      <c r="F31" s="239">
+      <c r="D31" s="237"/>
+      <c r="F31" s="236">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.15113729788983282</v>
       </c>
-      <c r="G31" s="240"/>
+      <c r="G31" s="237"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -38603,22 +38603,22 @@
       <c r="B33" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C33" s="239">
+      <c r="C33" s="236">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-0.2474056992258277</v>
       </c>
-      <c r="D33" s="240"/>
-      <c r="F33" s="239">
+      <c r="D33" s="237"/>
+      <c r="F33" s="236">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.25349794238683127</v>
       </c>
-      <c r="G33" s="240"/>
+      <c r="G33" s="237"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="227" t="s">
@@ -38645,22 +38645,22 @@
       <c r="B36" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C36" s="239">
+      <c r="C36" s="236">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-0.33159764979066247</v>
       </c>
-      <c r="D36" s="240"/>
-      <c r="F36" s="239">
+      <c r="D36" s="237"/>
+      <c r="F36" s="236">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21675455263551163</v>
       </c>
-      <c r="G36" s="240"/>
+      <c r="G36" s="237"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="227" t="s">
@@ -38687,22 +38687,22 @@
       <c r="B38" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C38" s="239">
+      <c r="C38" s="236">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>1.550202718817076E-3</v>
       </c>
-      <c r="D38" s="240"/>
-      <c r="F38" s="239">
+      <c r="D38" s="237"/>
+      <c r="F38" s="236">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>5.661089445213234E-2</v>
       </c>
-      <c r="G38" s="240"/>
+      <c r="G38" s="237"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="227" t="s">
@@ -38729,22 +38729,22 @@
       <c r="B40" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C40" s="239">
+      <c r="C40" s="236">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.19557882489819661</v>
       </c>
-      <c r="D40" s="240"/>
-      <c r="F40" s="239">
+      <c r="D40" s="237"/>
+      <c r="F40" s="236">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>7.9975007810059354E-2</v>
       </c>
-      <c r="G40" s="240"/>
+      <c r="G40" s="237"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="227" t="s">
@@ -38771,22 +38771,22 @@
       <c r="B42" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C42" s="239">
+      <c r="C42" s="236">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-0.31253806664926476</v>
       </c>
-      <c r="D42" s="240"/>
-      <c r="F42" s="239">
+      <c r="D42" s="237"/>
+      <c r="F42" s="236">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>5.0385535761765486E-2</v>
       </c>
-      <c r="G42" s="240"/>
+      <c r="G42" s="237"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="227" t="s">
@@ -38813,25 +38813,55 @@
       <c r="B44" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C44" s="239">
+      <c r="C44" s="236">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>3.2086096025055806E-2</v>
       </c>
-      <c r="D44" s="240"/>
-      <c r="F44" s="239">
+      <c r="D44" s="237"/>
+      <c r="F44" s="236">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.16254456746106211</v>
       </c>
-      <c r="G44" s="240"/>
+      <c r="G44" s="237"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -38840,36 +38870,6 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Fixed the EV/x valuations
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46326320-F300-6946-897C-CE5AA581779D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4BF1AB-0D5E-6C4A-8414-8E4E638DF49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="3" activeTab="12" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="8" activeTab="18" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -117,7 +117,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="5">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -128,7 +128,28 @@
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
         </ext>
       </extLst>
     </bk>
@@ -138,19 +159,28 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="5">
     <bk>
       <rc t="2" v="0"/>
     </bk>
     <bk>
       <rc t="2" v="1"/>
     </bk>
+    <bk>
+      <rc t="2" v="2"/>
+    </bk>
+    <bk>
+      <rc t="2" v="3"/>
+    </bk>
+    <bk>
+      <rc t="2" v="4"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="406">
   <si>
     <t>Ticker</t>
   </si>
@@ -2287,6 +2317,9 @@
     <xf numFmtId="10" fontId="23" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="23" fillId="12" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2294,9 +2327,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -15370,7 +15400,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1mou2&amp;q=XNAS%3aAAPL&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -15389,11 +15419,9 @@
     <v>Powered by Refinitiv</v>
     <v>317.39999999999998</v>
     <v>201.5</v>
-    <v>1.0868</v>
-    <v>14.25</v>
-    <v>4.8406999999999999E-2</v>
-    <v>-0.1893</v>
-    <v>-6.1339999999999995E-4</v>
+    <v>1.0903</v>
+    <v>-0.4</v>
+    <v>-1.2790000000000002E-3</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15401,35 +15429,49 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>309.42</v>
+    <v>315.48</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46205.999965821095</v>
+    <v>46210.767967233594</v>
     <v>0</v>
-    <v>293.68</v>
-    <v>4532959916800</v>
+    <v>310.14999999999998</v>
+    <v>4586275033600</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>294.12</v>
-    <v>35.752499999999998</v>
-    <v>294.38</v>
-    <v>308.63</v>
-    <v>308.44069999999999</v>
+    <v>315</v>
+    <v>37.924199999999999</v>
+    <v>312.66000000000003</v>
+    <v>312.26</v>
     <v>14687360000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>75400626</v>
-    <v>64811799</v>
+    <v>25322976</v>
+    <v>66025371</v>
     <v>1977</v>
   </rv>
   <rv s="2">
     <v>1</v>
   </rv>
+  <rv s="3">
+    <v>12</v>
+    <v>Price (Extended hours)</v>
+    <v>0</v>
+  </rv>
+  <rv s="3">
+    <v>12</v>
+    <v>Change (extended hours)</v>
+    <v>0</v>
+  </rv>
+  <rv s="3">
+    <v>12</v>
+    <v>Change % (extended hours)</v>
+    <v>0</v>
+  </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a33knm&amp;q=10+Y+TSY+YLD+NDX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="3">
+  <rv s="4">
     <v>5</v>
     <v>10 Y TSY YLD NDX</v>
     <v>6</v>
@@ -15443,28 +15485,28 @@
     <v>Powered by Refinitiv</v>
     <v>46.87</v>
     <v>39.47</v>
-    <v>0.1</v>
-    <v>2.235E-3</v>
+    <v>-0.06</v>
+    <v>-1.338E-3</v>
     <v>US</v>
-    <v>45.05</v>
+    <v>44.91</v>
     <v>Index</v>
-    <v>3</v>
-    <v>44.53</v>
+    <v>6</v>
+    <v>44.57</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>45.03</v>
-    <v>44.75</v>
+    <v>44.57</v>
     <v>44.85</v>
+    <v>44.79</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
   <rv s="2">
-    <v>4</v>
+    <v>7</v>
   </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
   <s t="_hyperlink">
     <k n="Address" t="s"/>
     <k n="Text" t="s"/>
@@ -15486,8 +15528,6 @@
     <k n="Beta"/>
     <k n="Change"/>
     <k n="Change (%)"/>
-    <k n="Change (Extended hours)"/>
-    <k n="Change % (Extended hours)"/>
     <k n="Currency" t="s"/>
     <k n="Description" t="s"/>
     <k n="Employees"/>
@@ -15508,7 +15548,6 @@
     <k n="P/E"/>
     <k n="Previous close"/>
     <k n="Price"/>
-    <k n="Price (Extended hours)"/>
     <k n="Shares outstanding"/>
     <k n="Ticker symbol" t="s"/>
     <k n="UniqueName" t="s"/>
@@ -15518,6 +15557,11 @@
   </s>
   <s t="_linkedentity">
     <k n="%cvi" t="r"/>
+  </s>
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="field" t="s"/>
+    <k n="subType" t="i"/>
   </s>
   <s t="_linkedentitycore">
     <k n="_Display" t="spb"/>
@@ -15553,7 +15597,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="2">
-    <a count="45">
+    <a count="42">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -15564,16 +15608,13 @@
       <v t="s">Name</v>
       <v t="s">_SubLabel</v>
       <v t="s">Price</v>
-      <v t="s">Price (Extended hours)</v>
       <v t="s">Exchange</v>
       <v t="s">Official name</v>
       <v t="s">Last trade time</v>
       <v t="s">Ticker symbol</v>
       <v t="s">Exchange abbreviation</v>
       <v t="s">Change</v>
-      <v t="s">Change (Extended hours)</v>
       <v t="s">Change (%)</v>
-      <v t="s">Change % (Extended hours)</v>
       <v t="s">Currency</v>
       <v t="s">Previous close</v>
       <v t="s">Open</v>
@@ -15667,19 +15708,13 @@
       <v>8</v>
       <v>9</v>
       <v>4</v>
-      <v>1</v>
-      <v>1</v>
-      <v>5</v>
     </spb>
     <spb s="4">
-      <v>at close</v>
+      <v>Real-Time Nasdaq Last Sale</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq</v>
+      <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
-      <v>Delayed 15 minutes</v>
-      <v>from close</v>
-      <v>from close</v>
     </spb>
     <spb s="0">
       <v>1</v>
@@ -15751,9 +15786,6 @@
     <k n="Year incorporated" t="i"/>
     <k n="`%EntityServiceId" t="i"/>
     <k n="Shares outstanding" t="i"/>
-    <k n="Price (Extended hours)" t="i"/>
-    <k n="Change (Extended hours)" t="i"/>
-    <k n="Change % (Extended hours)" t="i"/>
   </s>
   <s>
     <k n="Price" t="s"/>
@@ -15761,9 +15793,6 @@
     <k n="Change (%)" t="s"/>
     <k n="ExchangeID" t="s"/>
     <k n="Last trade time" t="s"/>
-    <k n="Price (Extended hours)" t="s"/>
-    <k n="Change (Extended hours)" t="s"/>
-    <k n="Change % (Extended hours)" t="s"/>
   </s>
   <s>
     <k n="UniqueName" t="spb"/>
@@ -16248,18 +16277,18 @@
   <sheetData>
     <row r="1" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="232" t="s">
+      <c r="B2" s="233" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="233"/>
-      <c r="E2" s="232" t="s">
+      <c r="C2" s="234"/>
+      <c r="E2" s="233" t="s">
         <v>286</v>
       </c>
-      <c r="F2" s="233"/>
-      <c r="H2" s="232" t="s">
+      <c r="F2" s="234"/>
+      <c r="H2" s="233" t="s">
         <v>327</v>
       </c>
-      <c r="I2" s="233"/>
+      <c r="I2" s="234"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="182" t="s">
@@ -16274,7 +16303,7 @@
       </c>
       <c r="F3" s="184">
         <f ca="1">Statement!AC143</f>
-        <v>4549206.2</v>
+        <v>4602712.3999999994</v>
       </c>
       <c r="H3" s="182" t="str">
         <f>'AVG target price'!B5</f>
@@ -16282,7 +16311,7 @@
       </c>
       <c r="I3" s="208">
         <f ca="1">'AVG target price'!C5</f>
-        <v>119.09057177167055</v>
+        <v>118.91617564595006</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16298,7 +16327,7 @@
       </c>
       <c r="F4" s="185">
         <f ca="1">Statement!AC144</f>
-        <v>4487322.2</v>
+        <v>4540828.3999999994</v>
       </c>
       <c r="H4" s="182" t="str">
         <f>'AVG target price'!B6</f>
@@ -16306,7 +16335,7 @@
       </c>
       <c r="I4" s="208">
         <f ca="1">'AVG target price'!C6</f>
-        <v>190.96664389474685</v>
+        <v>195.0721164457571</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16315,7 +16344,7 @@
       </c>
       <c r="C5" s="205" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
       <c r="E5" s="182" t="s">
         <v>242</v>
@@ -16337,16 +16366,16 @@
       <c r="B6" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="205" cm="1">
-        <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>308.44069999999999</v>
+      <c r="C6" s="205" t="e" cm="1" vm="2">
+        <f t="array" ref="C6">_FV(C3,"Price (Extended hours)",TRUE)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E6" s="182" t="s">
         <v>236</v>
       </c>
       <c r="F6" s="187">
         <f ca="1">Statement!AC140</f>
-        <v>37.319226118500609</v>
+        <v>37.758162031438935</v>
       </c>
       <c r="H6" s="182" t="str">
         <f>'AVG target price'!B8</f>
@@ -16354,7 +16383,7 @@
       </c>
       <c r="I6" s="208">
         <f ca="1">'AVG target price'!C8</f>
-        <v>122.01885943396663</v>
+        <v>126.15828009353453</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16363,14 +16392,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>14.25</v>
+        <v>-0.4</v>
       </c>
       <c r="E7" s="183" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="188">
         <f ca="1">Statement!AC141</f>
-        <v>10.143370156077635</v>
+        <v>10.262672990107257</v>
       </c>
       <c r="H7" s="181" t="str">
         <f>'AVG target price'!B9</f>
@@ -16378,23 +16407,23 @@
       </c>
       <c r="I7" s="209">
         <f ca="1">'AVG target price'!C9</f>
-        <v>142.69087684668344</v>
+        <v>144.70850111789787</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B8" s="182" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="6" cm="1">
-        <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-0.1893</v>
+      <c r="C8" s="6" t="e" cm="1" vm="3">
+        <f t="array" ref="C8">_FV(C3,"Change (extended hours)",TRUE)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E8" s="182" t="s">
         <v>264</v>
       </c>
       <c r="F8" s="189">
         <f ca="1">Statement!AC151</f>
-        <v>2.5433228328933518E-2</v>
+        <v>2.5137568882209544E-2</v>
       </c>
       <c r="H8" s="181" t="str">
         <f>'AVG target price'!B11</f>
@@ -16402,7 +16431,7 @@
       </c>
       <c r="I8" s="210">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.53766362036521587</v>
+        <v>-0.53657688747230559</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16411,30 +16440,30 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>4.8406999999999999E-2</v>
+        <v>-1.2790000000000002E-3</v>
       </c>
       <c r="E9" s="182" t="s">
         <v>287</v>
       </c>
       <c r="F9" s="189">
         <f ca="1">Statement!AC152</f>
-        <v>2.6795839678579528E-2</v>
+        <v>2.648433997309934E-2</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B10" s="182" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="73" cm="1">
-        <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-6.1339999999999995E-4</v>
+      <c r="C10" s="73" t="e" cm="1" vm="4">
+        <f t="array" ref="C10">_FV(C3,"Change % (extended hours)",TRUE)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E10" s="182" t="s">
         <v>292</v>
       </c>
       <c r="F10" s="189">
         <f ca="1">Statement!AC154</f>
-        <v>1.7188932873607708E-2</v>
+        <v>1.6989112767506396E-2</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -16450,7 +16479,7 @@
       </c>
       <c r="F11" s="190">
         <f ca="1">Statement!AC153</f>
-        <v>3.3697307455529276E-3</v>
+        <v>3.3305578684429643E-3</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16475,7 +16504,7 @@
       </c>
       <c r="C13" s="206" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.0868</v>
+        <v>1.0903</v>
       </c>
       <c r="E13" s="182" t="s">
         <v>101</v>
@@ -16491,7 +16520,7 @@
       </c>
       <c r="C14" s="207" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>64811799</v>
+        <v>66025371</v>
       </c>
       <c r="E14" s="183" t="s">
         <v>102</v>
@@ -16507,7 +16536,7 @@
       </c>
       <c r="F15" s="189">
         <f ca="1">Statement!AC166</f>
-        <v>1.3603252365214836E-2</v>
+        <v>1.344511553665617E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16520,10 +16549,10 @@
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="234" t="s">
+      <c r="B17" s="235" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="234"/>
+      <c r="C17" s="235"/>
       <c r="E17" s="181" t="s">
         <v>295</v>
       </c>
@@ -16596,14 +16625,14 @@
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="234" t="s">
+      <c r="B25" s="235" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="234"/>
-      <c r="E25" s="232" t="s">
+      <c r="C25" s="235"/>
+      <c r="E25" s="233" t="s">
         <v>342</v>
       </c>
-      <c r="F25" s="233"/>
+      <c r="F25" s="234"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="181" t="s">
@@ -16612,12 +16641,12 @@
       <c r="C26" s="167">
         <v>0.21</v>
       </c>
-      <c r="E26" s="182" t="e" vm="2">
+      <c r="E26" s="182" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
       <c r="F26" s="216" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>44.85</v>
+        <v>44.79</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16632,7 +16661,7 @@
       </c>
       <c r="F27" s="217">
         <f ca="1">F26/1000</f>
-        <v>4.4850000000000001E-2</v>
+        <v>4.4789999999999996E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -16652,15 +16681,15 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B33" s="235" t="s">
+      <c r="B33" s="232" t="s">
         <v>337</v>
       </c>
-      <c r="C33" s="235"/>
-      <c r="D33" s="235"/>
-      <c r="E33" s="235"/>
-      <c r="F33" s="235"/>
-      <c r="G33" s="235"/>
-      <c r="H33" s="235"/>
+      <c r="C33" s="232"/>
+      <c r="D33" s="232"/>
+      <c r="E33" s="232"/>
+      <c r="F33" s="232"/>
+      <c r="G33" s="232"/>
+      <c r="H33" s="232"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
@@ -16673,24 +16702,24 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="235"/>
-      <c r="C39" s="235"/>
-      <c r="D39" s="235"/>
-      <c r="E39" s="235"/>
-      <c r="F39" s="235"/>
-      <c r="G39" s="235"/>
-      <c r="H39" s="235"/>
+      <c r="B39" s="232"/>
+      <c r="C39" s="232"/>
+      <c r="D39" s="232"/>
+      <c r="E39" s="232"/>
+      <c r="F39" s="232"/>
+      <c r="G39" s="232"/>
+      <c r="H39" s="232"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B42" s="235" t="s">
+      <c r="B42" s="232" t="s">
         <v>340</v>
       </c>
-      <c r="C42" s="235"/>
-      <c r="D42" s="235"/>
-      <c r="E42" s="235"/>
-      <c r="F42" s="235"/>
-      <c r="G42" s="235"/>
-      <c r="H42" s="235"/>
+      <c r="C42" s="232"/>
+      <c r="D42" s="232"/>
+      <c r="E42" s="232"/>
+      <c r="F42" s="232"/>
+      <c r="G42" s="232"/>
+      <c r="H42" s="232"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="41" t="s">
@@ -16705,24 +16734,24 @@
       </c>
     </row>
     <row r="49" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="235"/>
-      <c r="C49" s="235"/>
-      <c r="D49" s="235"/>
-      <c r="E49" s="235"/>
-      <c r="F49" s="235"/>
-      <c r="G49" s="235"/>
-      <c r="H49" s="235"/>
+      <c r="B49" s="232"/>
+      <c r="C49" s="232"/>
+      <c r="D49" s="232"/>
+      <c r="E49" s="232"/>
+      <c r="F49" s="232"/>
+      <c r="G49" s="232"/>
+      <c r="H49" s="232"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="235" t="s">
+      <c r="B52" s="232" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="235"/>
-      <c r="D52" s="235"/>
-      <c r="E52" s="235"/>
-      <c r="F52" s="235"/>
-      <c r="G52" s="235"/>
-      <c r="H52" s="235"/>
+      <c r="C52" s="232"/>
+      <c r="D52" s="232"/>
+      <c r="E52" s="232"/>
+      <c r="F52" s="232"/>
+      <c r="G52" s="232"/>
+      <c r="H52" s="232"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" s="41" t="s">
@@ -16737,13 +16766,13 @@
       </c>
     </row>
     <row r="59" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="235"/>
-      <c r="C59" s="235"/>
-      <c r="D59" s="235"/>
-      <c r="E59" s="235"/>
-      <c r="F59" s="235"/>
-      <c r="G59" s="235"/>
-      <c r="H59" s="235"/>
+      <c r="B59" s="232"/>
+      <c r="C59" s="232"/>
+      <c r="D59" s="232"/>
+      <c r="E59" s="232"/>
+      <c r="F59" s="232"/>
+      <c r="G59" s="232"/>
+      <c r="H59" s="232"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -16828,36 +16857,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
       <c r="O2" s="5"/>
-      <c r="S2" s="235" t="s">
+      <c r="S2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="235"/>
-      <c r="U2" s="235"/>
-      <c r="V2" s="235"/>
-      <c r="W2" s="235"/>
-      <c r="X2" s="235"/>
-      <c r="Y2" s="235"/>
-      <c r="Z2" s="235"/>
-      <c r="AA2" s="235" t="s">
+      <c r="T2" s="232"/>
+      <c r="U2" s="232"/>
+      <c r="V2" s="232"/>
+      <c r="W2" s="232"/>
+      <c r="X2" s="232"/>
+      <c r="Y2" s="232"/>
+      <c r="Z2" s="232"/>
+      <c r="AA2" s="232" t="s">
         <v>111</v>
       </c>
-      <c r="AB2" s="235"/>
-      <c r="AC2" s="235"/>
+      <c r="AB2" s="232"/>
+      <c r="AC2" s="232"/>
       <c r="AE2" s="85" t="s">
         <v>112</v>
       </c>
@@ -18228,35 +18257,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
-      <c r="P2" s="235" t="s">
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="P2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="Q2" s="235"/>
-      <c r="R2" s="235"/>
-      <c r="S2" s="235"/>
-      <c r="T2" s="235"/>
-      <c r="U2" s="235"/>
-      <c r="V2" s="235"/>
-      <c r="W2" s="235"/>
-      <c r="X2" s="235" t="s">
+      <c r="Q2" s="232"/>
+      <c r="R2" s="232"/>
+      <c r="S2" s="232"/>
+      <c r="T2" s="232"/>
+      <c r="U2" s="232"/>
+      <c r="V2" s="232"/>
+      <c r="W2" s="232"/>
+      <c r="X2" s="232" t="s">
         <v>111</v>
       </c>
-      <c r="Y2" s="235"/>
-      <c r="Z2" s="235"/>
+      <c r="Y2" s="232"/>
+      <c r="Z2" s="232"/>
       <c r="AB2" s="85" t="s">
         <v>112</v>
       </c>
@@ -19487,20 +19516,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -20943,20 +20972,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
       <c r="S2" s="246"/>
       <c r="T2" s="246"/>
       <c r="U2" s="246"/>
@@ -22037,10 +22066,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="232" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="235"/>
+      <c r="C4" s="232"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -22057,7 +22086,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22066,7 +22095,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4549206.2</v>
+        <v>4602712.3999999994</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22084,7 +22113,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>4.4850000000000001E-2</v>
+        <v>4.4789999999999996E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22093,7 +22122,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.0868</v>
+        <v>1.0903</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22125,10 +22154,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="235" t="s">
+      <c r="B15" s="232" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="235"/>
+      <c r="C15" s="232"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -22136,7 +22165,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.8280646015858892E-2</v>
+        <v>1.8071975320172701E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22145,7 +22174,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98171935398414112</v>
+        <v>0.98192802467982732</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22163,7 +22192,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>9.3756000000000006E-2</v>
+        <v>9.3853500000000006E-2</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22172,7 +22201,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.2713619283529725E-2</v>
+        <v>9.282125587767473E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22217,20 +22246,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -22423,7 +22452,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1928325.9958641303</v>
+        <v>1925475.7505601391</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22477,23 +22506,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>96413.15957738203</v>
+        <v>96403.663436936506</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>93193.951001053298</v>
+        <v>93175.593771222775</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>90396.562769008087</v>
+        <v>90369.85477873635</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>87472.742554731027</v>
+        <v>87438.285402272217</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88239.749402833404</v>
+        <v>88196.302428934941</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22512,14 +22541,14 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1237794.8626094162</v>
+        <v>1235356.7292032014</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="235" t="s">
+      <c r="B13" s="232" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="235"/>
+      <c r="C13" s="232"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -22535,14 +22564,14 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2713619283529725E-2</v>
+        <v>9.282125587767473E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="235" t="s">
+      <c r="B18" s="232" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="235"/>
+      <c r="C18" s="232"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -22550,7 +22579,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>455716.16530500783</v>
+        <v>455583.69981810276</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22559,7 +22588,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1237794.8626094162</v>
+        <v>1235356.7292032014</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22568,7 +22597,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1693511.027914424</v>
+        <v>1690940.429021304</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22595,7 +22624,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1755395.027914424</v>
+        <v>1752824.429021304</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22613,7 +22642,7 @@
       </c>
       <c r="C26" s="142">
         <f ca="1">C24/C25</f>
-        <v>119.09057177167055</v>
+        <v>118.91617564595006</v>
       </c>
     </row>
   </sheetData>
@@ -22634,7 +22663,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D33819-10E3-B843-9B8A-30FFCAB234A7}">
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="83" customWidth="1"/>
@@ -22656,20 +22685,20 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -23601,10 +23630,10 @@
       <c r="N36" s="91"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B37" s="235" t="s">
+      <c r="B37" s="232" t="s">
         <v>202</v>
       </c>
-      <c r="C37" s="235"/>
+      <c r="C37" s="232"/>
       <c r="N37" s="91"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
@@ -23622,7 +23651,7 @@
       </c>
       <c r="C39" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2713619283529725E-2</v>
+        <v>9.282125587767473E-2</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -23635,182 +23664,227 @@
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B41" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C41" s="24">
+        <f>(C38*C40)</f>
+        <v>4332575.051406119</v>
+      </c>
+    </row>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B42" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="C42" s="24">
+        <f ca="1">C41/(1+C39)^5-G30+G31</f>
+        <v>2813478.9964104597</v>
+      </c>
+    </row>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B43" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C43" s="88">
+        <f>Statement!AC105</f>
+        <v>146595</v>
+      </c>
+    </row>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B44" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="88">
+        <f>Statement!AC106</f>
+        <v>84711</v>
+      </c>
+    </row>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B45" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C45" s="64">
+        <f ca="1">C42+C43-C44</f>
+        <v>2875362.9964104597</v>
+      </c>
+    </row>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B46" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C46" s="88">
+        <f>Statement!AC77</f>
+        <v>14740</v>
+      </c>
+    </row>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B47" s="141" t="s">
+        <v>206</v>
+      </c>
+      <c r="C47" s="142">
+        <f ca="1">C45/C46</f>
+        <v>195.0721164457571</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B49" s="232" t="s">
+        <v>207</v>
+      </c>
+      <c r="C49" s="232"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B50" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C50" s="64">
+        <f>L6</f>
+        <v>594236.0514889753</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B51" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C51" s="135">
+        <f>Overview!C29</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B52" s="39" t="s">
+        <v>209</v>
+      </c>
+      <c r="C52" s="105">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B53" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="C41" s="24">
+      <c r="C53" s="24">
         <f>L18</f>
         <v>13302.3529680093</v>
       </c>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B42" s="1" t="s">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B54" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C54" s="24">
+        <f>(C50*C52)/C53</f>
+        <v>223.35749657148918</v>
+      </c>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B55" s="141" t="s">
+        <v>206</v>
+      </c>
+      <c r="C55" s="142">
+        <f>C54/(1+C51)^5</f>
+        <v>138.68743228634972</v>
+      </c>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B57" s="232" t="s">
+        <v>321</v>
+      </c>
+      <c r="C57" s="232"/>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B58" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C58" s="64">
+        <f>L8</f>
+        <v>137466.23756646831</v>
+      </c>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B59" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C59" s="135">
+        <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
+        <v>9.282125587767473E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B60" s="39" t="s">
+        <v>350</v>
+      </c>
+      <c r="C60" s="105">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B61" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C42" s="24">
-        <f>(C38*C40)</f>
-        <v>4332575.051406119</v>
-      </c>
-    </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B43" s="1" t="s">
+      <c r="C61" s="24">
+        <f>(C58*C60)</f>
+        <v>2749324.7513293661</v>
+      </c>
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B62" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="C43" s="24">
-        <f ca="1">C42/(1+C39)^5-G30+G31</f>
-        <v>2814848.3310085684</v>
-      </c>
-    </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B44" s="1" t="s">
+      <c r="C62" s="24">
+        <f ca="1">C61/(1+C59)^5-G30+G31</f>
+        <v>1797689.0485786989</v>
+      </c>
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B63" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C63" s="88">
+        <f>Statement!AC105</f>
+        <v>146595</v>
+      </c>
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B64" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C64" s="88">
+        <f>Statement!AC106</f>
+        <v>84711</v>
+      </c>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B65" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C65" s="64">
+        <f ca="1">C62+C63-C64</f>
+        <v>1859573.0485786989</v>
+      </c>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B66" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C44" s="88">
+      <c r="C66" s="88">
         <f>Statement!AC77</f>
         <v>14740</v>
       </c>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B45" s="141" t="s">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B67" s="141" t="s">
         <v>206</v>
       </c>
-      <c r="C45" s="142">
-        <f ca="1">C43/C44</f>
-        <v>190.96664389474685</v>
-      </c>
-    </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B47" s="235" t="s">
-        <v>207</v>
-      </c>
-      <c r="C47" s="235"/>
-    </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B48" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="C48" s="64">
-        <f>L6</f>
-        <v>594236.0514889753</v>
-      </c>
-    </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B49" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="C49" s="135">
-        <f>Overview!C29</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B50" s="39" t="s">
-        <v>209</v>
-      </c>
-      <c r="C50" s="105">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B51" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C51" s="24">
-        <f>L18</f>
-        <v>13302.3529680093</v>
-      </c>
-    </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B52" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C52" s="24">
-        <f>(C48*C50)/C51</f>
-        <v>223.35749657148918</v>
-      </c>
-    </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B53" s="141" t="s">
-        <v>206</v>
-      </c>
-      <c r="C53" s="142">
-        <f>C52/(1+C49)^5</f>
-        <v>138.68743228634972</v>
-      </c>
-    </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B55" s="235" t="s">
-        <v>321</v>
-      </c>
-      <c r="C55" s="235"/>
-    </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B56" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C56" s="64">
-        <f>L8</f>
-        <v>137466.23756646831</v>
-      </c>
-    </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B57" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="C57" s="135">
-        <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2713619283529725E-2</v>
-      </c>
-    </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B58" s="39" t="s">
-        <v>350</v>
-      </c>
-      <c r="C58" s="105">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B59" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C59" s="24">
-        <f>(C56*C58)</f>
-        <v>2749324.7513293661</v>
-      </c>
-    </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B60" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="C60" s="24">
-        <f ca="1">C59/(1+C57)^5-G30+G31</f>
-        <v>1798557.9880566681</v>
-      </c>
-    </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B61" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C61" s="88">
-        <f>Statement!AC77</f>
-        <v>14740</v>
-      </c>
-    </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B62" s="141" t="s">
-        <v>206</v>
-      </c>
-      <c r="C62" s="142">
-        <f ca="1">C60/C61</f>
-        <v>122.01885943396663</v>
+      <c r="C67" s="142">
+        <f ca="1">C65/C66</f>
+        <v>126.15828009353453</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B57:C57"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
@@ -23854,10 +23928,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="232" t="s">
         <v>212</v>
       </c>
-      <c r="C4" s="235"/>
+      <c r="C4" s="232"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -23866,7 +23940,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>119.09057177167055</v>
+        <v>118.91617564595006</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -23874,8 +23948,8 @@
         <v>214</v>
       </c>
       <c r="C6" s="133">
-        <f ca="1">Multiples!C45</f>
-        <v>190.96664389474685</v>
+        <f ca="1">Multiples!C47</f>
+        <v>195.0721164457571</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -23883,7 +23957,7 @@
         <v>215</v>
       </c>
       <c r="C7" s="133">
-        <f>Multiples!C53</f>
+        <f>Multiples!C55</f>
         <v>138.68743228634972</v>
       </c>
     </row>
@@ -23892,8 +23966,8 @@
         <v>322</v>
       </c>
       <c r="C8" s="133">
-        <f ca="1">Multiples!C62</f>
-        <v>122.01885943396663</v>
+        <f ca="1">Multiples!C67</f>
+        <v>126.15828009353453</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -23902,7 +23976,7 @@
       </c>
       <c r="C9" s="142">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>142.69087684668344</v>
+        <v>144.70850111789787</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -23911,7 +23985,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C5</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -23920,7 +23994,7 @@
       </c>
       <c r="C11" s="151">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.53766362036521587</v>
+        <v>-0.53657688747230559</v>
       </c>
     </row>
   </sheetData>
@@ -23985,20 +24059,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -24173,7 +24247,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>5255703.4594641058</v>
+        <v>5247935.0405677995</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -24227,23 +24301,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>145028.49718044625</v>
+        <v>145014.21270948954</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>164576.82354290391</v>
+        <v>164544.405402648</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>186760.06008510161</v>
+        <v>186704.88115224056</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>211933.36517336537</v>
+        <v>211849.88064936845</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>240499.76881159769</v>
+        <v>240381.35293611235</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -24262,7 +24336,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3373642.6078765481</v>
+        <v>3366997.4108480564</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -24278,7 +24352,7 @@
       </c>
       <c r="C15" s="153">
         <f ca="1">Overview!C5</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -24287,7 +24361,7 @@
       </c>
       <c r="C16" s="153">
         <f ca="1">C36</f>
-        <v>298.51740468917842</v>
+        <v>298.04426660978521</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -24326,7 +24400,7 @@
       </c>
       <c r="C21" s="219">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.2713619283529725E-2</v>
+        <v>9.282125587767473E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -24344,7 +24418,7 @@
       </c>
       <c r="C23" s="158">
         <f ca="1">C15*C22</f>
-        <v>4532848.8099999996</v>
+        <v>4586162.62</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -24371,7 +24445,7 @@
       </c>
       <c r="C26" s="159">
         <f ca="1">C23+C25-C24</f>
-        <v>4470964.8099999996</v>
+        <v>4524278.62</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -24387,7 +24461,7 @@
       </c>
       <c r="C29" s="158">
         <f ca="1">SUM(H10:L10)</f>
-        <v>948798.51479341486</v>
+        <v>948494.73284985893</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -24396,7 +24470,7 @@
       </c>
       <c r="C30" s="158">
         <f ca="1">L11</f>
-        <v>3373642.6078765481</v>
+        <v>3366997.4108480564</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -24405,7 +24479,7 @@
       </c>
       <c r="C31" s="161">
         <f ca="1">C29+C30</f>
-        <v>4322441.1226699632</v>
+        <v>4315492.1436979156</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -24432,7 +24506,7 @@
       </c>
       <c r="C34" s="161">
         <f ca="1">C31+C32-C33</f>
-        <v>4384325.1226699632</v>
+        <v>4377376.1436979156</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -24450,7 +24524,7 @@
       </c>
       <c r="C36" s="164">
         <f ca="1">C34/C35</f>
-        <v>298.51740468917842</v>
+        <v>298.04426660978521</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -31305,7 +31379,7 @@
       <c r="AA114" s="68"/>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31352,7 +31426,7 @@
       <c r="AA115" s="68"/>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32266,7 +32340,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>37.319226118500609</v>
+        <v>37.758162031438935</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32303,7 +32377,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.143370156077635</v>
+        <v>10.262672990107257</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32340,7 +32414,7 @@
       <c r="AA142" s="49"/>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>42.565557746664034</v>
+        <v>43.066199209322853</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32377,7 +32451,7 @@
       <c r="AA143" s="49"/>
       <c r="AC143" s="143">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4549206.2</v>
+        <v>4602712.3999999994</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -32414,7 +32488,7 @@
       <c r="AA144" s="49"/>
       <c r="AC144" s="143">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4487322.2</v>
+        <v>4540828.3999999994</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -32451,7 +32525,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="180">
         <f ca="1">AC144/AC5</f>
-        <v>9.9399750134015008</v>
+        <v>10.05849788012635</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -32488,7 +32562,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="180">
         <f ca="1">AC144/AC11</f>
-        <v>30.450186610208597</v>
+        <v>30.813270360870209</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -32623,7 +32697,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="89">AC143/AC147</f>
-        <v>39.318642016922929</v>
+        <v>39.781094372563757</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -32660,7 +32734,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="89"/>
-        <v>38.824496757041281</v>
+        <v>39.28743460634071</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -32697,7 +32771,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="92">AC147/AC143</f>
-        <v>2.5433228328933518E-2</v>
+        <v>2.5137568882209544E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -32734,7 +32808,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.6795839678579528E-2</v>
+        <v>2.648433997309934E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -32771,7 +32845,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="151">
         <f ca="1">AC81/AC115</f>
-        <v>3.3697307455529276E-3</v>
+        <v>3.3305578684429643E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -32808,7 +32882,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="151">
         <f ca="1">-AC62/AC143</f>
-        <v>1.7188932873607708E-2</v>
+        <v>1.6989112767506396E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -32845,7 +32919,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="151">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>2.0607111631915035E-2</v>
+        <v>2.0367555444046431E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33348,7 +33422,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="151">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.3603252365214836E-2</v>
+        <v>1.344511553665617E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35345,15 +35419,15 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="232" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="235"/>
-      <c r="E4" s="235" t="s">
+      <c r="C4" s="232"/>
+      <c r="E4" s="232" t="s">
         <v>239</v>
       </c>
-      <c r="F4" s="235"/>
-      <c r="G4" s="235"/>
+      <c r="F4" s="232"/>
+      <c r="G4" s="232"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
@@ -35361,7 +35435,7 @@
       </c>
       <c r="C5" s="169">
         <f ca="1">Overview!C5</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -35377,7 +35451,7 @@
       </c>
       <c r="C6" s="170">
         <f ca="1">Statement!AC143</f>
-        <v>4549206.2</v>
+        <v>4602712.3999999994</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -35397,7 +35471,7 @@
       </c>
       <c r="C7" s="170">
         <f ca="1">Statement!AC144</f>
-        <v>4487322.2</v>
+        <v>4540828.3999999994</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -35417,7 +35491,7 @@
       </c>
       <c r="C8" s="171">
         <f ca="1">Statement!AC140</f>
-        <v>37.319226118500609</v>
+        <v>37.758162031438935</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>242</v>
@@ -35437,7 +35511,7 @@
       </c>
       <c r="C9" s="171">
         <f ca="1">Statement!AC141</f>
-        <v>10.143370156077635</v>
+        <v>10.262672990107257</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>243</v>
@@ -35457,7 +35531,7 @@
       </c>
       <c r="C10" s="171">
         <f ca="1">Statement!AC142</f>
-        <v>42.565557746664034</v>
+        <v>43.066199209322853</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -35477,7 +35551,7 @@
       </c>
       <c r="C11" s="171">
         <f ca="1">Statement!AC145</f>
-        <v>9.9399750134015008</v>
+        <v>10.05849788012635</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -35486,18 +35560,18 @@
       </c>
       <c r="C12" s="171">
         <f ca="1">Statement!AC146</f>
-        <v>30.450186610208597</v>
+        <v>30.813270360870209</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="235" t="s">
+      <c r="B15" s="232" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="235"/>
-      <c r="E15" s="235" t="s">
+      <c r="C15" s="232"/>
+      <c r="E15" s="232" t="s">
         <v>245</v>
       </c>
-      <c r="F15" s="235"/>
+      <c r="F15" s="232"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
@@ -35548,14 +35622,14 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="235" t="s">
+      <c r="B21" s="232" t="s">
         <v>244</v>
       </c>
-      <c r="C21" s="235"/>
-      <c r="E21" s="235" t="s">
+      <c r="C21" s="232"/>
+      <c r="E21" s="232" t="s">
         <v>248</v>
       </c>
-      <c r="F21" s="235"/>
+      <c r="F21" s="232"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
@@ -35624,14 +35698,14 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B29" s="235" t="s">
+      <c r="B29" s="232" t="s">
         <v>249</v>
       </c>
-      <c r="C29" s="235"/>
-      <c r="E29" s="235" t="s">
+      <c r="C29" s="232"/>
+      <c r="E29" s="232" t="s">
         <v>255</v>
       </c>
-      <c r="F29" s="235"/>
+      <c r="F29" s="232"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -35707,14 +35781,14 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B37" s="235" t="s">
+      <c r="B37" s="232" t="s">
         <v>267</v>
       </c>
-      <c r="C37" s="235"/>
-      <c r="E37" s="235" t="s">
+      <c r="C37" s="232"/>
+      <c r="E37" s="232" t="s">
         <v>270</v>
       </c>
-      <c r="F37" s="235"/>
+      <c r="F37" s="232"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
@@ -35722,7 +35796,7 @@
       </c>
       <c r="C38" s="172">
         <f ca="1">Statement!AC152</f>
-        <v>2.6795839678579528E-2</v>
+        <v>2.648433997309934E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>269</v>
@@ -35738,7 +35812,7 @@
       </c>
       <c r="C39" s="212">
         <f ca="1">Statement!AC151</f>
-        <v>2.5433228328933518E-2</v>
+        <v>2.5137568882209544E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>271</v>
@@ -35754,7 +35828,7 @@
       </c>
       <c r="C40" s="172">
         <f ca="1">Statement!AC153</f>
-        <v>3.3697307455529276E-3</v>
+        <v>3.3305578684429643E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>272</v>
@@ -35770,7 +35844,7 @@
       </c>
       <c r="C41" s="172">
         <f ca="1">Statement!AC154</f>
-        <v>1.7188932873607708E-2</v>
+        <v>1.6989112767506396E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -35779,18 +35853,18 @@
       </c>
       <c r="C42" s="172">
         <f ca="1">Statement!AC155</f>
-        <v>2.0607111631915035E-2</v>
+        <v>2.0367555444046431E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B45" s="235" t="s">
+      <c r="B45" s="232" t="s">
         <v>278</v>
       </c>
-      <c r="C45" s="235"/>
-      <c r="E45" s="235" t="s">
+      <c r="C45" s="232"/>
+      <c r="E45" s="232" t="s">
         <v>284</v>
       </c>
-      <c r="F45" s="235"/>
+      <c r="F45" s="232"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
@@ -35823,18 +35897,18 @@
       </c>
       <c r="F48" s="172">
         <f ca="1">Statement!AC166</f>
-        <v>1.3603252365214836E-2</v>
+        <v>1.344511553665617E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B51" s="235" t="s">
+      <c r="B51" s="232" t="s">
         <v>281</v>
       </c>
-      <c r="C51" s="235"/>
-      <c r="E51" s="235" t="s">
+      <c r="C51" s="232"/>
+      <c r="E51" s="232" t="s">
         <v>302</v>
       </c>
-      <c r="F51" s="235"/>
+      <c r="F51" s="232"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
@@ -36002,7 +36076,7 @@
       </c>
       <c r="I6" s="169">
         <f ca="1">Statement!AC114</f>
-        <v>308.63</v>
+        <v>312.26</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36031,7 +36105,7 @@
       </c>
       <c r="I7" s="170">
         <f ca="1">Statement!AC143</f>
-        <v>4549206.2</v>
+        <v>4602712.3999999994</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36060,7 +36134,7 @@
       </c>
       <c r="I8" s="170">
         <f ca="1">Statement!AC144</f>
-        <v>4487322.2</v>
+        <v>4540828.3999999994</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36089,7 +36163,7 @@
       </c>
       <c r="I9" s="171">
         <f ca="1">Statement!AC140</f>
-        <v>37.319226118500609</v>
+        <v>37.758162031438935</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36118,7 +36192,7 @@
       </c>
       <c r="I10" s="171">
         <f ca="1">Statement!AC141</f>
-        <v>10.143370156077635</v>
+        <v>10.262672990107257</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36147,7 +36221,7 @@
       </c>
       <c r="I11" s="171">
         <f ca="1">Statement!AC142</f>
-        <v>42.565557746664034</v>
+        <v>43.066199209322853</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36176,7 +36250,7 @@
       </c>
       <c r="I12" s="171">
         <f ca="1">Statement!AC145</f>
-        <v>9.9399750134015008</v>
+        <v>10.05849788012635</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36205,7 +36279,7 @@
       </c>
       <c r="I13" s="171">
         <f ca="1">Statement!AC146</f>
-        <v>30.450186610208597</v>
+        <v>30.813270360870209</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -36978,7 +37052,7 @@
       </c>
       <c r="I51" s="172">
         <f ca="1">Statement!AC152</f>
-        <v>2.6795839678579528E-2</v>
+        <v>2.648433997309934E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37007,7 +37081,7 @@
       </c>
       <c r="I52" s="172">
         <f ca="1">Statement!AC151</f>
-        <v>2.5433228328933518E-2</v>
+        <v>2.5137568882209544E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37036,7 +37110,7 @@
       </c>
       <c r="I53" s="172">
         <f ca="1">Statement!AC153</f>
-        <v>3.3697307455529276E-3</v>
+        <v>3.3305578684429643E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37065,7 +37139,7 @@
       </c>
       <c r="I54" s="172">
         <f ca="1">Statement!AC154</f>
-        <v>1.7188932873607708E-2</v>
+        <v>1.6989112767506396E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37094,7 +37168,7 @@
       </c>
       <c r="I55" s="172">
         <f ca="1">Statement!AC155</f>
-        <v>2.0607111631915035E-2</v>
+        <v>2.0367555444046431E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37330,7 +37404,7 @@
       </c>
       <c r="I68" s="193">
         <f ca="1">Statement!AC166</f>
-        <v>1.3603252365214836E-2</v>
+        <v>1.344511553665617E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated all models with DDM and added MU
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD5252E-72F5-7649-9C41-6EE97B78816D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B3157A-2698-C74D-BA44-79D191A8B7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -32,10 +32,12 @@
     <sheet name="DCF" sheetId="11" r:id="rId17"/>
     <sheet name="Multiples" sheetId="12" r:id="rId18"/>
     <sheet name="AVG target price" sheetId="13" r:id="rId19"/>
-    <sheet name="Reverse DCF" sheetId="14" r:id="rId20"/>
+    <sheet name="DDM" sheetId="21" r:id="rId20"/>
+    <sheet name="Reverse DCF" sheetId="14" r:id="rId21"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId21"/>
+    <externalReference r:id="rId22"/>
+    <externalReference r:id="rId23"/>
   </externalReferences>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -150,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="417">
   <si>
     <t>Ticker</t>
   </si>
@@ -1368,6 +1370,39 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Manual Cost of Equity</t>
+  </si>
+  <si>
+    <t>DDM price</t>
+  </si>
+  <si>
+    <t>Dividend discount model</t>
+  </si>
+  <si>
+    <t>Dividend per share</t>
+  </si>
+  <si>
+    <t>Ratios</t>
+  </si>
+  <si>
+    <t>Payout</t>
+  </si>
+  <si>
+    <t>DDM valuation</t>
+  </si>
+  <si>
+    <t>Latest dividend</t>
+  </si>
+  <si>
+    <t>Year 1 growth rate</t>
+  </si>
+  <si>
+    <t>Year 1 dividend</t>
+  </si>
+  <si>
+    <t>Perpetual dividend growth</t>
   </si>
 </sst>
 </file>
@@ -1980,7 +2015,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="250">
+  <cellXfs count="255">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -2287,6 +2322,9 @@
     <xf numFmtId="10" fontId="23" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="23" fillId="12" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2296,15 +2334,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2312,6 +2341,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2341,6 +2376,11 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="39" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="39" fontId="17" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="39" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15260,6 +15300,95 @@
 </externalLink>
 </file>
 
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Overview"/>
+      <sheetName val="Financials -&gt;"/>
+      <sheetName val="Statement"/>
+      <sheetName val="Analysis -&gt;"/>
+      <sheetName val="Basic"/>
+      <sheetName val="Yearly Analysis"/>
+      <sheetName val="Quarter analysis"/>
+      <sheetName val="Graphs Year"/>
+      <sheetName val="Graphs Quarter"/>
+      <sheetName val="Forecast -&gt;"/>
+      <sheetName val="Revenue"/>
+      <sheetName val="COGS &amp; OpEx"/>
+      <sheetName val="WC &amp; Investments"/>
+      <sheetName val="FCF &amp; Other"/>
+      <sheetName val="Valuation -&gt;"/>
+      <sheetName val="WACC"/>
+      <sheetName val="DCF"/>
+      <sheetName val="Multiples"/>
+      <sheetName val="AVG target price"/>
+      <sheetName val="DDM"/>
+      <sheetName val="Reverse DCF"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10">
+        <row r="5">
+          <cell r="C5">
+            <v>2021</v>
+          </cell>
+          <cell r="D5">
+            <v>2022</v>
+          </cell>
+          <cell r="E5">
+            <v>2023</v>
+          </cell>
+          <cell r="F5">
+            <v>2024</v>
+          </cell>
+          <cell r="G5">
+            <v>2025</v>
+          </cell>
+          <cell r="H5">
+            <v>2026</v>
+          </cell>
+          <cell r="I5">
+            <v>2027</v>
+          </cell>
+          <cell r="J5">
+            <v>2028</v>
+          </cell>
+          <cell r="K5">
+            <v>2029</v>
+          </cell>
+          <cell r="L5">
+            <v>2030</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="adi dumitras" id="{A0F62302-F8D3-B346-B5DF-839B413AE710}" userId="b24535bb88af1c42" providerId="Windows Live"/>
@@ -15389,11 +15518,11 @@
     <v>Powered by Refinitiv</v>
     <v>317.39999999999998</v>
     <v>201.5</v>
-    <v>1.0904</v>
+    <v>1.0931999999999999</v>
     <v>-0.9</v>
     <v>-2.846E-3</v>
-    <v>-0.21809999999999999</v>
-    <v>-6.9169999999999995E-4</v>
+    <v>-0.35</v>
+    <v>-1.1100000000000001E-3</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15404,21 +15533,21 @@
     <v>316.91000000000003</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46213.888557071092</v>
+    <v>46213.99998719844</v>
     <v>0</v>
     <v>312.17</v>
     <v>4631218355200</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
     <v>314.72000000000003</v>
-    <v>38.2958</v>
+    <v>38.405000000000001</v>
     <v>316.22000000000003</v>
     <v>315.32</v>
-    <v>315.1019</v>
+    <v>314.97000000000003</v>
     <v>14687360000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>32478188</v>
+    <v>34132321</v>
     <v>64766433</v>
     <v>1977</v>
   </rv>
@@ -15443,17 +15572,17 @@
     <v>Powered by Refinitiv</v>
     <v>46.87</v>
     <v>39.47</v>
-    <v>-0.3</v>
-    <v>-6.5659999999999998E-3</v>
+    <v>0.3</v>
+    <v>6.6090000000000003E-3</v>
     <v>US</v>
-    <v>45.81</v>
+    <v>45.71</v>
     <v>Index</v>
     <v>3</v>
-    <v>45.29</v>
+    <v>45.39</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>45.77</v>
+    <v>45.41</v>
+    <v>45.39</v>
     <v>45.69</v>
-    <v>45.39</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -15675,9 +15804,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq Last Sale</v>
+      <v>Source: Nasdaq</v>
       <v>GMT</v>
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>Delayed 15 minutes</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -16248,18 +16377,18 @@
   <sheetData>
     <row r="1" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="232" t="s">
+      <c r="B2" s="233" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="233"/>
-      <c r="E2" s="232" t="s">
+      <c r="C2" s="234"/>
+      <c r="E2" s="233" t="s">
         <v>286</v>
       </c>
-      <c r="F2" s="233"/>
-      <c r="H2" s="232" t="s">
+      <c r="F2" s="234"/>
+      <c r="H2" s="233" t="s">
         <v>327</v>
       </c>
-      <c r="I2" s="233"/>
+      <c r="I2" s="234"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="182" t="s">
@@ -16282,7 +16411,7 @@
       </c>
       <c r="I3" s="208">
         <f ca="1">'AVG target price'!C5</f>
-        <v>117.94784406159961</v>
+        <v>117.28589507926682</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16306,7 +16435,7 @@
       </c>
       <c r="I4" s="208">
         <f ca="1">'AVG target price'!C6</f>
-        <v>194.55224664880012</v>
+        <v>194.19286803829158</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16339,7 +16468,7 @@
       </c>
       <c r="C6" s="205" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>315.1019</v>
+        <v>314.97000000000003</v>
       </c>
       <c r="E6" s="182" t="s">
         <v>236</v>
@@ -16354,7 +16483,7 @@
       </c>
       <c r="I6" s="208">
         <f ca="1">'AVG target price'!C8</f>
-        <v>125.82838600438804</v>
+        <v>125.60033490377322</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16378,7 +16507,7 @@
       </c>
       <c r="I7" s="209">
         <f ca="1">'AVG target price'!C9</f>
-        <v>144.25397725028435</v>
+        <v>143.94163257692031</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -16387,7 +16516,7 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-0.21809999999999999</v>
+        <v>-0.35</v>
       </c>
       <c r="E8" s="182" t="s">
         <v>264</v>
@@ -16402,7 +16531,7 @@
       </c>
       <c r="I8" s="210">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.5425156119171497</v>
+        <v>-0.54350617602143758</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16427,7 +16556,7 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-6.9169999999999995E-4</v>
+        <v>-1.1100000000000001E-3</v>
       </c>
       <c r="E10" s="182" t="s">
         <v>292</v>
@@ -16436,6 +16565,13 @@
         <f ca="1">Statement!AC154</f>
         <v>1.6824243158637408E-2</v>
       </c>
+      <c r="H10" s="181" t="s">
+        <v>407</v>
+      </c>
+      <c r="I10" s="209">
+        <f>DDM!C26</f>
+        <v>13.26</v>
+      </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B11" s="182" t="s">
@@ -16475,7 +16611,7 @@
       </c>
       <c r="C13" s="206" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.0904</v>
+        <v>1.0931999999999999</v>
       </c>
       <c r="E13" s="182" t="s">
         <v>101</v>
@@ -16520,10 +16656,10 @@
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="234" t="s">
+      <c r="B17" s="235" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="234"/>
+      <c r="C17" s="235"/>
       <c r="E17" s="181" t="s">
         <v>295</v>
       </c>
@@ -16596,14 +16732,14 @@
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="234" t="s">
+      <c r="B25" s="235" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="234"/>
-      <c r="E25" s="232" t="s">
+      <c r="C25" s="235"/>
+      <c r="E25" s="233" t="s">
         <v>342</v>
       </c>
-      <c r="F25" s="233"/>
+      <c r="F25" s="234"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="181" t="s">
@@ -16617,7 +16753,7 @@
       </c>
       <c r="F26" s="216" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>45.39</v>
+        <v>45.69</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16632,7 +16768,7 @@
       </c>
       <c r="F27" s="217">
         <f ca="1">F26/1000</f>
-        <v>4.539E-2</v>
+        <v>4.5689999999999995E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -16645,22 +16781,22 @@
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="181" t="s">
-        <v>348</v>
+        <v>406</v>
       </c>
       <c r="C29" s="218">
         <v>0.1</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B33" s="235" t="s">
+      <c r="B33" s="232" t="s">
         <v>337</v>
       </c>
-      <c r="C33" s="235"/>
-      <c r="D33" s="235"/>
-      <c r="E33" s="235"/>
-      <c r="F33" s="235"/>
-      <c r="G33" s="235"/>
-      <c r="H33" s="235"/>
+      <c r="C33" s="232"/>
+      <c r="D33" s="232"/>
+      <c r="E33" s="232"/>
+      <c r="F33" s="232"/>
+      <c r="G33" s="232"/>
+      <c r="H33" s="232"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
@@ -16673,24 +16809,24 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="235"/>
-      <c r="C39" s="235"/>
-      <c r="D39" s="235"/>
-      <c r="E39" s="235"/>
-      <c r="F39" s="235"/>
-      <c r="G39" s="235"/>
-      <c r="H39" s="235"/>
+      <c r="B39" s="232"/>
+      <c r="C39" s="232"/>
+      <c r="D39" s="232"/>
+      <c r="E39" s="232"/>
+      <c r="F39" s="232"/>
+      <c r="G39" s="232"/>
+      <c r="H39" s="232"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B42" s="235" t="s">
+      <c r="B42" s="232" t="s">
         <v>340</v>
       </c>
-      <c r="C42" s="235"/>
-      <c r="D42" s="235"/>
-      <c r="E42" s="235"/>
-      <c r="F42" s="235"/>
-      <c r="G42" s="235"/>
-      <c r="H42" s="235"/>
+      <c r="C42" s="232"/>
+      <c r="D42" s="232"/>
+      <c r="E42" s="232"/>
+      <c r="F42" s="232"/>
+      <c r="G42" s="232"/>
+      <c r="H42" s="232"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="41" t="s">
@@ -16705,24 +16841,24 @@
       </c>
     </row>
     <row r="49" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="235"/>
-      <c r="C49" s="235"/>
-      <c r="D49" s="235"/>
-      <c r="E49" s="235"/>
-      <c r="F49" s="235"/>
-      <c r="G49" s="235"/>
-      <c r="H49" s="235"/>
+      <c r="B49" s="232"/>
+      <c r="C49" s="232"/>
+      <c r="D49" s="232"/>
+      <c r="E49" s="232"/>
+      <c r="F49" s="232"/>
+      <c r="G49" s="232"/>
+      <c r="H49" s="232"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="235" t="s">
+      <c r="B52" s="232" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="235"/>
-      <c r="D52" s="235"/>
-      <c r="E52" s="235"/>
-      <c r="F52" s="235"/>
-      <c r="G52" s="235"/>
-      <c r="H52" s="235"/>
+      <c r="C52" s="232"/>
+      <c r="D52" s="232"/>
+      <c r="E52" s="232"/>
+      <c r="F52" s="232"/>
+      <c r="G52" s="232"/>
+      <c r="H52" s="232"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" s="41" t="s">
@@ -16737,28 +16873,28 @@
       </c>
     </row>
     <row r="59" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="235"/>
-      <c r="C59" s="235"/>
-      <c r="D59" s="235"/>
-      <c r="E59" s="235"/>
-      <c r="F59" s="235"/>
-      <c r="G59" s="235"/>
-      <c r="H59" s="235"/>
+      <c r="B59" s="232"/>
+      <c r="C59" s="232"/>
+      <c r="D59" s="232"/>
+      <c r="E59" s="232"/>
+      <c r="F59" s="232"/>
+      <c r="G59" s="232"/>
+      <c r="H59" s="232"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="E25:F25"/>
     <mergeCell ref="B52:H52"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B42:H42"/>
     <mergeCell ref="B49:H49"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="E25:F25"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C10">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
@@ -16828,36 +16964,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
       <c r="O2" s="5"/>
-      <c r="S2" s="235" t="s">
+      <c r="S2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="235"/>
-      <c r="U2" s="235"/>
-      <c r="V2" s="235"/>
-      <c r="W2" s="235"/>
-      <c r="X2" s="235"/>
-      <c r="Y2" s="235"/>
-      <c r="Z2" s="235"/>
-      <c r="AA2" s="235" t="s">
+      <c r="T2" s="232"/>
+      <c r="U2" s="232"/>
+      <c r="V2" s="232"/>
+      <c r="W2" s="232"/>
+      <c r="X2" s="232"/>
+      <c r="Y2" s="232"/>
+      <c r="Z2" s="232"/>
+      <c r="AA2" s="232" t="s">
         <v>111</v>
       </c>
-      <c r="AB2" s="235"/>
-      <c r="AC2" s="235"/>
+      <c r="AB2" s="232"/>
+      <c r="AC2" s="232"/>
       <c r="AE2" s="85" t="s">
         <v>112</v>
       </c>
@@ -18228,35 +18364,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
-      <c r="P2" s="235" t="s">
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="P2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="Q2" s="235"/>
-      <c r="R2" s="235"/>
-      <c r="S2" s="235"/>
-      <c r="T2" s="235"/>
-      <c r="U2" s="235"/>
-      <c r="V2" s="235"/>
-      <c r="W2" s="235"/>
-      <c r="X2" s="235" t="s">
+      <c r="Q2" s="232"/>
+      <c r="R2" s="232"/>
+      <c r="S2" s="232"/>
+      <c r="T2" s="232"/>
+      <c r="U2" s="232"/>
+      <c r="V2" s="232"/>
+      <c r="W2" s="232"/>
+      <c r="X2" s="232" t="s">
         <v>111</v>
       </c>
-      <c r="Y2" s="235"/>
-      <c r="Z2" s="235"/>
+      <c r="Y2" s="232"/>
+      <c r="Z2" s="232"/>
       <c r="AB2" s="85" t="s">
         <v>112</v>
       </c>
@@ -19487,20 +19623,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -20893,12 +21029,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -20906,6 +21036,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -20943,20 +21079,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
       <c r="S2" s="246"/>
       <c r="T2" s="246"/>
       <c r="U2" s="246"/>
@@ -21965,16 +22101,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="C25:L25"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="S2:Z2"/>
     <mergeCell ref="AA2:AC2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="S4:AC4"/>
     <mergeCell ref="C13:L13"/>
     <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="C25:L25"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22037,10 +22173,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="232" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="235"/>
+      <c r="C4" s="232"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -22084,7 +22220,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>4.539E-2</v>
+        <v>4.5689999999999995E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22093,7 +22229,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.0904</v>
+        <v>1.0931999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22125,10 +22261,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="235" t="s">
+      <c r="B15" s="232" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="235"/>
+      <c r="C15" s="232"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -22163,7 +22299,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>9.4458E-2</v>
+        <v>9.4883999999999996E-2</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22172,7 +22308,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.3424773517315624E-2</v>
+        <v>9.3843148229620532E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22217,20 +22353,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -22423,7 +22559,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1909649.2314645126</v>
+        <v>1898829.6907627422</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22477,23 +22613,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>96350.45327303739</v>
+        <v>96313.601012058483</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>93072.765306374349</v>
+        <v>93001.581709908671</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>90220.297978009301</v>
+        <v>90116.814797603191</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>87245.398338495695</v>
+        <v>87111.995913326784</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>87953.170485233975</v>
+        <v>87785.096824080858</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22512,14 +22648,14 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1221825.1360868276</v>
+        <v>1212581.0032114149</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="235" t="s">
+      <c r="B13" s="232" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="235"/>
+      <c r="C13" s="232"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -22535,14 +22671,14 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.3424773517315624E-2</v>
+        <v>9.3843148229620532E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="235" t="s">
+      <c r="B18" s="232" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="235"/>
+      <c r="C18" s="232"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -22550,7 +22686,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>454842.08538115071</v>
+        <v>454329.090256978</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22559,7 +22695,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1221825.1360868276</v>
+        <v>1212581.0032114149</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22568,7 +22704,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1676667.2214679783</v>
+        <v>1666910.093468393</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22595,7 +22731,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1738551.2214679783</v>
+        <v>1728794.093468393</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22613,7 +22749,7 @@
       </c>
       <c r="C26" s="142">
         <f ca="1">C24/C25</f>
-        <v>117.94784406159961</v>
+        <v>117.28589507926682</v>
       </c>
     </row>
   </sheetData>
@@ -22656,20 +22792,20 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
       <c r="G2" s="244"/>
       <c r="H2" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -23601,10 +23737,10 @@
       <c r="N36" s="91"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B37" s="235" t="s">
+      <c r="B37" s="232" t="s">
         <v>202</v>
       </c>
-      <c r="C37" s="235"/>
+      <c r="C37" s="232"/>
       <c r="N37" s="91"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
@@ -23622,7 +23758,7 @@
       </c>
       <c r="C39" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.3424773517315624E-2</v>
+        <v>9.3843148229620532E-2</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -23648,7 +23784,7 @@
       </c>
       <c r="C42" s="24">
         <f ca="1">C41/(1+C39)^5-G30+G31</f>
-        <v>2805816.1156033138</v>
+        <v>2800518.8748844177</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.2">
@@ -23675,7 +23811,7 @@
       </c>
       <c r="C45" s="64">
         <f ca="1">C42+C43-C44</f>
-        <v>2867700.1156033138</v>
+        <v>2862402.8748844177</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -23693,14 +23829,14 @@
       </c>
       <c r="C47" s="142">
         <f ca="1">C45/C46</f>
-        <v>194.55224664880012</v>
+        <v>194.19286803829158</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B49" s="235" t="s">
+      <c r="B49" s="232" t="s">
         <v>207</v>
       </c>
-      <c r="C49" s="235"/>
+      <c r="C49" s="232"/>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
@@ -23716,7 +23852,7 @@
         <v>348</v>
       </c>
       <c r="C51" s="135">
-        <f>Overview!C29</f>
+        <f>IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
         <v>0.1</v>
       </c>
     </row>
@@ -23756,10 +23892,10 @@
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B57" s="235" t="s">
+      <c r="B57" s="232" t="s">
         <v>321</v>
       </c>
-      <c r="C57" s="235"/>
+      <c r="C57" s="232"/>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B58" s="1" t="s">
@@ -23776,7 +23912,7 @@
       </c>
       <c r="C59" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.3424773517315624E-2</v>
+        <v>9.3843148229620532E-2</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -23802,7 +23938,7 @@
       </c>
       <c r="C62" s="24">
         <f ca="1">C61/(1+C59)^5-G30+G31</f>
-        <v>1792826.4097046796</v>
+        <v>1789464.9364816172</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -23829,7 +23965,7 @@
       </c>
       <c r="C65" s="64">
         <f ca="1">C62+C63-C64</f>
-        <v>1854710.4097046796</v>
+        <v>1851348.9364816172</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -23847,7 +23983,7 @@
       </c>
       <c r="C67" s="142">
         <f ca="1">C65/C66</f>
-        <v>125.82838600438804</v>
+        <v>125.60033490377322</v>
       </c>
     </row>
   </sheetData>
@@ -23899,10 +24035,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="232" t="s">
         <v>212</v>
       </c>
-      <c r="C4" s="235"/>
+      <c r="C4" s="232"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -23911,7 +24047,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>117.94784406159961</v>
+        <v>117.28589507926682</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -23920,7 +24056,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C47</f>
-        <v>194.55224664880012</v>
+        <v>194.19286803829158</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -23938,7 +24074,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C67</f>
-        <v>125.82838600438804</v>
+        <v>125.60033490377322</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -23947,7 +24083,7 @@
       </c>
       <c r="C9" s="142">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>144.25397725028435</v>
+        <v>143.94163257692031</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -23965,7 +24101,7 @@
       </c>
       <c r="C11" s="151">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.5425156119171497</v>
+        <v>-0.54350617602143758</v>
       </c>
     </row>
   </sheetData>
@@ -23998,6 +24134,477 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{272A8DA5-299F-1343-8F22-D98E787B4AC7}">
+  <dimension ref="A1:N26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2" style="83" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" style="1"/>
+    <col min="4" max="4" width="10.83203125" style="1" customWidth="1"/>
+    <col min="5" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
+    <col min="9" max="12" width="10.83203125" style="1"/>
+    <col min="13" max="14" width="9.5" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="83" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4"/>
+      <c r="B1" s="82" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2" s="4"/>
+      <c r="C2" s="232" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="244"/>
+      <c r="H2" s="245" t="s">
+        <v>111</v>
+      </c>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+    </row>
+    <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="86"/>
+      <c r="B4" s="60"/>
+      <c r="C4" s="241" t="s">
+        <v>191</v>
+      </c>
+      <c r="D4" s="241"/>
+      <c r="E4" s="241"/>
+      <c r="F4" s="241"/>
+      <c r="G4" s="241"/>
+      <c r="H4" s="241"/>
+      <c r="I4" s="241"/>
+      <c r="J4" s="241"/>
+      <c r="K4" s="241"/>
+      <c r="L4" s="241"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B5" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="12">
+        <f>[2]Revenue!C5</f>
+        <v>2021</v>
+      </c>
+      <c r="D5" s="12">
+        <f>[2]Revenue!D5</f>
+        <v>2022</v>
+      </c>
+      <c r="E5" s="12">
+        <f>[2]Revenue!E5</f>
+        <v>2023</v>
+      </c>
+      <c r="F5" s="12">
+        <f>[2]Revenue!F5</f>
+        <v>2024</v>
+      </c>
+      <c r="G5" s="12">
+        <f>[2]Revenue!G5</f>
+        <v>2025</v>
+      </c>
+      <c r="H5" s="12">
+        <f>[2]Revenue!H5</f>
+        <v>2026</v>
+      </c>
+      <c r="I5" s="12">
+        <f>[2]Revenue!I5</f>
+        <v>2027</v>
+      </c>
+      <c r="J5" s="12">
+        <f>[2]Revenue!J5</f>
+        <v>2028</v>
+      </c>
+      <c r="K5" s="12">
+        <f>[2]Revenue!K5</f>
+        <v>2029</v>
+      </c>
+      <c r="L5" s="12">
+        <f>[2]Revenue!L5</f>
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B6" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" s="250">
+        <f>Statement!M25</f>
+        <v>5.61</v>
+      </c>
+      <c r="D6" s="250">
+        <f>Statement!N25</f>
+        <v>6.11</v>
+      </c>
+      <c r="E6" s="250">
+        <f>Statement!O25</f>
+        <v>6.13</v>
+      </c>
+      <c r="F6" s="250">
+        <f>Statement!P25</f>
+        <v>6.08</v>
+      </c>
+      <c r="G6" s="251">
+        <f>Statement!Q25</f>
+        <v>7.46</v>
+      </c>
+      <c r="H6" s="137"/>
+      <c r="I6" s="137"/>
+      <c r="J6" s="137"/>
+      <c r="K6" s="137"/>
+      <c r="L6" s="137"/>
+      <c r="N6" s="91"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B7" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="C7" s="250">
+        <f>Statement!M81</f>
+        <v>0.85</v>
+      </c>
+      <c r="D7" s="250">
+        <f>Statement!N81</f>
+        <v>0.9</v>
+      </c>
+      <c r="E7" s="250">
+        <f>Statement!O81</f>
+        <v>0.94</v>
+      </c>
+      <c r="F7" s="250">
+        <f>Statement!P81</f>
+        <v>0.98</v>
+      </c>
+      <c r="G7" s="251">
+        <f>Statement!Q81</f>
+        <v>1.02</v>
+      </c>
+      <c r="H7" s="137"/>
+      <c r="I7" s="137"/>
+      <c r="J7" s="137"/>
+      <c r="K7" s="137"/>
+      <c r="L7" s="137"/>
+      <c r="N7" s="91"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="N8" s="91"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C9" s="241" t="s">
+        <v>119</v>
+      </c>
+      <c r="D9" s="241"/>
+      <c r="E9" s="241"/>
+      <c r="F9" s="241"/>
+      <c r="G9" s="241"/>
+      <c r="H9" s="241"/>
+      <c r="I9" s="241"/>
+      <c r="J9" s="241"/>
+      <c r="K9" s="241"/>
+      <c r="L9" s="241"/>
+      <c r="N9" s="91"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B10" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="C10" s="12">
+        <f t="shared" ref="C10:L10" si="0">C5</f>
+        <v>2021</v>
+      </c>
+      <c r="D10" s="12">
+        <f t="shared" si="0"/>
+        <v>2022</v>
+      </c>
+      <c r="E10" s="12">
+        <f t="shared" si="0"/>
+        <v>2023</v>
+      </c>
+      <c r="F10" s="12">
+        <f t="shared" si="0"/>
+        <v>2024</v>
+      </c>
+      <c r="G10" s="12">
+        <f t="shared" si="0"/>
+        <v>2025</v>
+      </c>
+      <c r="H10" s="12">
+        <f t="shared" si="0"/>
+        <v>2026</v>
+      </c>
+      <c r="I10" s="12">
+        <f t="shared" si="0"/>
+        <v>2027</v>
+      </c>
+      <c r="J10" s="12">
+        <f t="shared" si="0"/>
+        <v>2028</v>
+      </c>
+      <c r="K10" s="12">
+        <f t="shared" si="0"/>
+        <v>2029</v>
+      </c>
+      <c r="L10" s="12">
+        <f t="shared" si="0"/>
+        <v>2030</v>
+      </c>
+      <c r="N10" s="91"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B11" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C11" s="137"/>
+      <c r="D11" s="95">
+        <f>(D6-C6)/C6</f>
+        <v>8.9126559714795009E-2</v>
+      </c>
+      <c r="E11" s="95">
+        <f>(E6-D6)/D6</f>
+        <v>3.2733224222585224E-3</v>
+      </c>
+      <c r="F11" s="95">
+        <f>(F6-E6)/E6</f>
+        <v>-8.1566068515497268E-3</v>
+      </c>
+      <c r="G11" s="96">
+        <f>(G6-F6)/F6</f>
+        <v>0.2269736842105263</v>
+      </c>
+      <c r="H11" s="137"/>
+      <c r="I11" s="137"/>
+      <c r="J11" s="137"/>
+      <c r="K11" s="137"/>
+      <c r="L11" s="137"/>
+      <c r="N11" s="91"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C12" s="137"/>
+      <c r="D12" s="95">
+        <f>IF(C7=0,
+IF(D7=0,0,IF(D7&gt;0,1,-1)),
+(D7-C7)/ABS(C7)
+)</f>
+        <v>5.8823529411764761E-2</v>
+      </c>
+      <c r="E12" s="95">
+        <f>IF(D7=0,
+IF(E7=0,0,IF(E7&gt;0,1,-1)),
+(E7-D7)/ABS(D7)
+)</f>
+        <v>4.4444444444444363E-2</v>
+      </c>
+      <c r="F12" s="95">
+        <f>IF(E7=0,
+IF(F7=0,0,IF(F7&gt;0,1,-1)),
+(F7-E7)/ABS(E7)
+)</f>
+        <v>4.2553191489361743E-2</v>
+      </c>
+      <c r="G12" s="96">
+        <f>IF(F7=0,
+IF(G7=0,0,IF(G7&gt;0,1,-1)),
+(G7-F7)/ABS(F7)
+)</f>
+        <v>4.0816326530612283E-2</v>
+      </c>
+      <c r="H12" s="137"/>
+      <c r="I12" s="137"/>
+      <c r="J12" s="137"/>
+      <c r="K12" s="137"/>
+      <c r="L12" s="137"/>
+      <c r="N12" s="91"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="N13" s="91"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C14" s="241" t="s">
+        <v>410</v>
+      </c>
+      <c r="D14" s="241"/>
+      <c r="E14" s="241"/>
+      <c r="F14" s="241"/>
+      <c r="G14" s="241"/>
+      <c r="H14" s="241"/>
+      <c r="I14" s="241"/>
+      <c r="J14" s="241"/>
+      <c r="K14" s="241"/>
+      <c r="L14" s="241"/>
+      <c r="N14" s="91"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B15" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="C15" s="12">
+        <f>C5</f>
+        <v>2021</v>
+      </c>
+      <c r="D15" s="12">
+        <f t="shared" ref="D15:L15" si="1">D5</f>
+        <v>2022</v>
+      </c>
+      <c r="E15" s="12">
+        <f t="shared" si="1"/>
+        <v>2023</v>
+      </c>
+      <c r="F15" s="12">
+        <f t="shared" si="1"/>
+        <v>2024</v>
+      </c>
+      <c r="G15" s="12">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="H15" s="12">
+        <f t="shared" si="1"/>
+        <v>2026</v>
+      </c>
+      <c r="I15" s="12">
+        <f t="shared" si="1"/>
+        <v>2027</v>
+      </c>
+      <c r="J15" s="12">
+        <f t="shared" si="1"/>
+        <v>2028</v>
+      </c>
+      <c r="K15" s="12">
+        <f t="shared" si="1"/>
+        <v>2029</v>
+      </c>
+      <c r="L15" s="12">
+        <f t="shared" si="1"/>
+        <v>2030</v>
+      </c>
+      <c r="N15" s="91"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B16" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="C16" s="95">
+        <f>C7/C6</f>
+        <v>0.15151515151515149</v>
+      </c>
+      <c r="D16" s="95">
+        <f t="shared" ref="D16:G16" si="2">D7/D6</f>
+        <v>0.14729950900163666</v>
+      </c>
+      <c r="E16" s="95">
+        <f t="shared" si="2"/>
+        <v>0.15334420880913541</v>
+      </c>
+      <c r="F16" s="95">
+        <f t="shared" si="2"/>
+        <v>0.16118421052631579</v>
+      </c>
+      <c r="G16" s="96">
+        <f t="shared" si="2"/>
+        <v>0.13672922252010725</v>
+      </c>
+      <c r="H16" s="137"/>
+      <c r="I16" s="137"/>
+      <c r="J16" s="137"/>
+      <c r="K16" s="137"/>
+      <c r="L16" s="137"/>
+      <c r="N16" s="91"/>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N17" s="91"/>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N18" s="91"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N19" s="91"/>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B20" s="232" t="s">
+        <v>412</v>
+      </c>
+      <c r="C20" s="232"/>
+      <c r="N20" s="91"/>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B21" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="C21" s="252">
+        <f>G7</f>
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B22" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="C22" s="253">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B23" s="39" t="s">
+        <v>415</v>
+      </c>
+      <c r="C23" s="254">
+        <f>C21*(1+C22)</f>
+        <v>1.0608</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B24" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C24" s="135">
+        <f>IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B25" s="39" t="s">
+        <v>416</v>
+      </c>
+      <c r="C25" s="253">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B26" s="141" t="s">
+        <v>206</v>
+      </c>
+      <c r="C26" s="142">
+        <f>C23/(C24-C25)</f>
+        <v>13.26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="C9:L9"/>
+    <mergeCell ref="C14:L14"/>
+    <mergeCell ref="B20:C20"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0116CE1A-CCEC-514B-9208-A0DCC7740441}">
   <dimension ref="A1:AB49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -24030,20 +24637,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
       <c r="G3" s="244"/>
       <c r="H3" s="245" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
       <c r="P3" s="246"/>
       <c r="Q3" s="246"/>
       <c r="R3" s="246"/>
@@ -24218,7 +24825,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>5204799.4445427703</v>
+        <v>5175310.5004440695</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -24272,23 +24879,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>144934.17187130061</v>
+        <v>144878.73723923485</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>164362.81440953349</v>
+        <v>164237.1069996765</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>186395.89554223133</v>
+        <v>186182.09841988026</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>211382.54415881552</v>
+        <v>211059.33004590889</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>239718.69039857667</v>
+        <v>239260.60119360726</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -24307,7 +24914,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3330116.6962249489</v>
+        <v>3304921.567788545</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -24332,7 +24939,7 @@
       </c>
       <c r="C16" s="153">
         <f ca="1">C36</f>
-        <v>295.41736315145408</v>
+        <v>293.62180443159616</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -24371,7 +24978,7 @@
       </c>
       <c r="C21" s="219">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.3424773517315624E-2</v>
+        <v>9.3843148229620532E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -24432,7 +25039,7 @@
       </c>
       <c r="C29" s="158">
         <f ca="1">SUM(H10:L10)</f>
-        <v>946794.11638045753</v>
+        <v>945617.87389830779</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -24441,7 +25048,7 @@
       </c>
       <c r="C30" s="158">
         <f ca="1">L11</f>
-        <v>3330116.6962249489</v>
+        <v>3304921.567788545</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -24450,7 +25057,7 @@
       </c>
       <c r="C31" s="161">
         <f ca="1">C29+C30</f>
-        <v>4276910.8126054062</v>
+        <v>4250539.4416868528</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -24477,7 +25084,7 @@
       </c>
       <c r="C34" s="161">
         <f ca="1">C31+C32-C33</f>
-        <v>4338794.8126054062</v>
+        <v>4312423.4416868528</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -24495,7 +25102,7 @@
       </c>
       <c r="C36" s="164">
         <f ca="1">C34/C35</f>
-        <v>295.41736315145408</v>
+        <v>293.62180443159616</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -24942,17 +25549,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C39:L39"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C39:L39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -35390,15 +35997,15 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="232" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="235"/>
-      <c r="E4" s="235" t="s">
+      <c r="C4" s="232"/>
+      <c r="E4" s="232" t="s">
         <v>239</v>
       </c>
-      <c r="F4" s="235"/>
-      <c r="G4" s="235"/>
+      <c r="F4" s="232"/>
+      <c r="G4" s="232"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
@@ -35535,14 +36142,14 @@
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="235" t="s">
+      <c r="B15" s="232" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="235"/>
-      <c r="E15" s="235" t="s">
+      <c r="C15" s="232"/>
+      <c r="E15" s="232" t="s">
         <v>245</v>
       </c>
-      <c r="F15" s="235"/>
+      <c r="F15" s="232"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
@@ -35593,14 +36200,14 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="235" t="s">
+      <c r="B21" s="232" t="s">
         <v>244</v>
       </c>
-      <c r="C21" s="235"/>
-      <c r="E21" s="235" t="s">
+      <c r="C21" s="232"/>
+      <c r="E21" s="232" t="s">
         <v>248</v>
       </c>
-      <c r="F21" s="235"/>
+      <c r="F21" s="232"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
@@ -35669,14 +36276,14 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B29" s="235" t="s">
+      <c r="B29" s="232" t="s">
         <v>249</v>
       </c>
-      <c r="C29" s="235"/>
-      <c r="E29" s="235" t="s">
+      <c r="C29" s="232"/>
+      <c r="E29" s="232" t="s">
         <v>255</v>
       </c>
-      <c r="F29" s="235"/>
+      <c r="F29" s="232"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -35752,14 +36359,14 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B37" s="235" t="s">
+      <c r="B37" s="232" t="s">
         <v>267</v>
       </c>
-      <c r="C37" s="235"/>
-      <c r="E37" s="235" t="s">
+      <c r="C37" s="232"/>
+      <c r="E37" s="232" t="s">
         <v>270</v>
       </c>
-      <c r="F37" s="235"/>
+      <c r="F37" s="232"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
@@ -35828,14 +36435,14 @@
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B45" s="235" t="s">
+      <c r="B45" s="232" t="s">
         <v>278</v>
       </c>
-      <c r="C45" s="235"/>
-      <c r="E45" s="235" t="s">
+      <c r="C45" s="232"/>
+      <c r="E45" s="232" t="s">
         <v>284</v>
       </c>
-      <c r="F45" s="235"/>
+      <c r="F45" s="232"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
@@ -35872,14 +36479,14 @@
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B51" s="235" t="s">
+      <c r="B51" s="232" t="s">
         <v>281</v>
       </c>
-      <c r="C51" s="235"/>
-      <c r="E51" s="235" t="s">
+      <c r="C51" s="232"/>
+      <c r="E51" s="232" t="s">
         <v>302</v>
       </c>
-      <c r="F51" s="235"/>
+      <c r="F51" s="232"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
@@ -38067,14 +38674,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="238" t="s">
+      <c r="C3" s="236" t="s">
         <v>312</v>
       </c>
-      <c r="D3" s="239"/>
-      <c r="F3" s="240" t="s">
+      <c r="D3" s="237"/>
+      <c r="F3" s="238" t="s">
         <v>313</v>
       </c>
-      <c r="G3" s="239"/>
+      <c r="G3" s="237"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38141,19 +38748,19 @@
       <c r="B7" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C7" s="236">
+      <c r="C7" s="239">
         <f>Statement!AA88</f>
         <v>-0.22657836890286318</v>
       </c>
-      <c r="D7" s="237"/>
-      <c r="F7" s="236">
+      <c r="D7" s="240"/>
+      <c r="F7" s="239">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16595182415922985</v>
       </c>
-      <c r="G7" s="237"/>
+      <c r="G7" s="240"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="204" t="s">
@@ -38180,19 +38787,19 @@
       <c r="B9" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C9" s="236">
+      <c r="C9" s="239">
         <f>Statement!AA89</f>
         <v>-0.24316672257631666</v>
       </c>
-      <c r="D9" s="237"/>
-      <c r="F9" s="236">
+      <c r="D9" s="240"/>
+      <c r="F9" s="239">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>0.11706805038421929</v>
       </c>
-      <c r="G9" s="237"/>
+      <c r="G9" s="240"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="204" t="s">
@@ -38219,19 +38826,19 @@
       <c r="B11" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C11" s="236">
+      <c r="C11" s="239">
         <f>Statement!AA90</f>
         <v>-0.2087215264838006</v>
       </c>
-      <c r="D11" s="237"/>
-      <c r="F11" s="236">
+      <c r="D11" s="240"/>
+      <c r="F11" s="239">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.22096418302984375</v>
       </c>
-      <c r="G11" s="237"/>
+      <c r="G11" s="240"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="204" t="s">
@@ -38258,19 +38865,19 @@
       <c r="B13" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C13" s="236">
+      <c r="C13" s="239">
         <f>Statement!AA93</f>
         <v>2.8129930899396048E-2</v>
       </c>
-      <c r="D13" s="237"/>
-      <c r="F13" s="236">
+      <c r="D13" s="240"/>
+      <c r="F13" s="239">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.23681110092944102</v>
       </c>
-      <c r="G13" s="237"/>
+      <c r="G13" s="240"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="204" t="s">
@@ -38297,19 +38904,19 @@
       <c r="B15" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C15" s="236">
+      <c r="C15" s="239">
         <f>Statement!AA94</f>
         <v>-0.29432470699284197</v>
       </c>
-      <c r="D15" s="237"/>
-      <c r="F15" s="236">
+      <c r="D15" s="240"/>
+      <c r="F15" s="239">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.21278177701172732</v>
       </c>
-      <c r="G15" s="237"/>
+      <c r="G15" s="240"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="204" t="s">
@@ -38336,19 +38943,19 @@
       <c r="B17" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C17" s="236">
+      <c r="C17" s="239">
         <f>Statement!AA96</f>
         <v>-0.29738461173005204</v>
       </c>
-      <c r="D17" s="237"/>
-      <c r="F17" s="236">
+      <c r="D17" s="240"/>
+      <c r="F17" s="239">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.19362389023405974</v>
       </c>
-      <c r="G17" s="237"/>
+      <c r="G17" s="240"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="204" t="s">
@@ -38375,22 +38982,22 @@
       <c r="B19" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C19" s="236">
+      <c r="C19" s="239">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-5.6718433490884537E-3</v>
       </c>
-      <c r="D19" s="237"/>
-      <c r="F19" s="236">
+      <c r="D19" s="240"/>
+      <c r="F19" s="239">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-2.1918172157279491E-2</v>
       </c>
-      <c r="G19" s="237"/>
+      <c r="G19" s="240"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="204" t="s">
@@ -38417,22 +39024,22 @@
       <c r="B21" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C21" s="236">
+      <c r="C21" s="239">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>-0.29225352112676062</v>
       </c>
-      <c r="D21" s="237"/>
-      <c r="F21" s="236">
+      <c r="D21" s="240"/>
+      <c r="F21" s="239">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.21818181818181812</v>
       </c>
-      <c r="G21" s="237"/>
+      <c r="G21" s="240"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -38480,22 +39087,22 @@
       <c r="B25" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C25" s="236">
+      <c r="C25" s="239">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>-0.22956141399989749</v>
       </c>
-      <c r="D25" s="237"/>
-      <c r="F25" s="236">
+      <c r="D25" s="240"/>
+      <c r="F25" s="239">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11851668113605358</v>
       </c>
-      <c r="G25" s="237"/>
+      <c r="G25" s="240"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -38522,22 +39129,22 @@
       <c r="B27" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C27" s="236">
+      <c r="C27" s="239">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>-0.26453625543962672</v>
       </c>
-      <c r="D27" s="237"/>
-      <c r="F27" s="236">
+      <c r="D27" s="240"/>
+      <c r="F27" s="239">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.14725607262615523</v>
       </c>
-      <c r="G27" s="237"/>
+      <c r="G27" s="240"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -38564,22 +39171,22 @@
       <c r="B29" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C29" s="236">
+      <c r="C29" s="239">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-0.19701480843061975</v>
       </c>
-      <c r="D29" s="237"/>
-      <c r="F29" s="236">
+      <c r="D29" s="240"/>
+      <c r="F29" s="239">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.28090238720159982</v>
       </c>
-      <c r="G29" s="237"/>
+      <c r="G29" s="240"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -38606,22 +39213,22 @@
       <c r="B31" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C31" s="236">
+      <c r="C31" s="239">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.10751088919579305</v>
       </c>
-      <c r="D31" s="237"/>
-      <c r="F31" s="236">
+      <c r="D31" s="240"/>
+      <c r="F31" s="239">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.15113729788983282</v>
       </c>
-      <c r="G31" s="237"/>
+      <c r="G31" s="240"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -38648,22 +39255,22 @@
       <c r="B33" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C33" s="236">
+      <c r="C33" s="239">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-0.2474056992258277</v>
       </c>
-      <c r="D33" s="237"/>
-      <c r="F33" s="236">
+      <c r="D33" s="240"/>
+      <c r="F33" s="239">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.25349794238683127</v>
       </c>
-      <c r="G33" s="237"/>
+      <c r="G33" s="240"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="227" t="s">
@@ -38690,22 +39297,22 @@
       <c r="B36" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C36" s="236">
+      <c r="C36" s="239">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-0.33159764979066247</v>
       </c>
-      <c r="D36" s="237"/>
-      <c r="F36" s="236">
+      <c r="D36" s="240"/>
+      <c r="F36" s="239">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21675455263551163</v>
       </c>
-      <c r="G36" s="237"/>
+      <c r="G36" s="240"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="227" t="s">
@@ -38732,22 +39339,22 @@
       <c r="B38" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C38" s="236">
+      <c r="C38" s="239">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>1.550202718817076E-3</v>
       </c>
-      <c r="D38" s="237"/>
-      <c r="F38" s="236">
+      <c r="D38" s="240"/>
+      <c r="F38" s="239">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>5.661089445213234E-2</v>
       </c>
-      <c r="G38" s="237"/>
+      <c r="G38" s="240"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="227" t="s">
@@ -38774,22 +39381,22 @@
       <c r="B40" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C40" s="236">
+      <c r="C40" s="239">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.19557882489819661</v>
       </c>
-      <c r="D40" s="237"/>
-      <c r="F40" s="236">
+      <c r="D40" s="240"/>
+      <c r="F40" s="239">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>7.9975007810059354E-2</v>
       </c>
-      <c r="G40" s="237"/>
+      <c r="G40" s="240"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="227" t="s">
@@ -38816,22 +39423,22 @@
       <c r="B42" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C42" s="236">
+      <c r="C42" s="239">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-0.31253806664926476</v>
       </c>
-      <c r="D42" s="237"/>
-      <c r="F42" s="236">
+      <c r="D42" s="240"/>
+      <c r="F42" s="239">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>5.0385535761765486E-2</v>
       </c>
-      <c r="G42" s="237"/>
+      <c r="G42" s="240"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="227" t="s">
@@ -38858,55 +39465,25 @@
       <c r="B44" s="203" t="s">
         <v>314</v>
       </c>
-      <c r="C44" s="236">
+      <c r="C44" s="239">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>3.2086096025055806E-2</v>
       </c>
-      <c r="D44" s="237"/>
-      <c r="F44" s="236">
+      <c r="D44" s="240"/>
+      <c r="F44" s="239">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.16254456746106211</v>
       </c>
-      <c r="G44" s="237"/>
+      <c r="G44" s="240"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -38915,6 +39492,36 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>